<commit_message>
docs(report): sửa nhãn biên của email - @Size không khai min nên không có min-1
Kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều hợp lệ, nên
gọi 6 là 'min' là sai. Ràng buộc email chỉ có @Size(max=150) - không khai min.

Sửa theo mẫu slide 29 (một trường mang nhiều điều kiện độc lập):
- email tách làm 2 dòng: điều kiện ĐỘ DÀI (có biên trên) và điều kiện
  ĐỊNH DẠNG (miền rời rạc, không có biên)
- 6 và 7 ký tự đổi nhãn thành 'giá trị ngắn hợp lệ', không phải min/min+1
- Robustness của email chỉ còn max+1 = 151

Đối chiếu: password có @Size(min=6) nên min-1 = 5 là giá trị không hợp lệ
thật; fullName có biên dưới do @NotBlank nên chuỗi rỗng chính là min-1.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>min = 6 ký tự</t>
+          <t>giá trị ngắn hợp lệ (không phải biên) = 6 ký tự</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>email · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>min+1 = 7 ký tự</t>
+          <t>giá trị ngắn hợp lệ (không phải biên) = 7 ký tự</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B8</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>email · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B9</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>B12</t>
+          <t>B10</t>
         </is>
       </c>
     </row>
@@ -1232,17 +1232,17 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>email · Robustness / Negative</t>
+          <t>email · Robustness</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>null = null</t>
+          <t>max+1 = 151 ký tự</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B11</t>
         </is>
       </c>
     </row>
@@ -1274,17 +1274,17 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>email · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>empty = rỗng</t>
+          <t>null = null</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1316,17 +1316,17 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>email · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>invalid = sai định dạng</t>
+          <t>empty = rỗng</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1358,17 +1358,17 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>email · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>max+1 = 151</t>
+          <t>invalid format = sai định dạng</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>B13</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -2403,20 +2403,19 @@
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>101</t>
+          <t>rỗng (= min−1), 101</t>
         </is>
       </c>
     </row>
     <row r="51" ht="62" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>email — điều kiện ĐỘ DÀI</t>
         </is>
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>đúng định dạng email,
-≤ 150 ký tự</t>
+          <t>≤ 150 ký tự</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -2426,52 +2425,94 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>sai định dạng
-&gt; 150 ký tự
-null</t>
+          <t>&gt; 150 ký tự</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>X8
-X9
-X10</t>
+          <t>X9</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>6, 7, 75, 149, 150</t>
+          <t>75, 149, 150
+(không có biên dưới)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>B8–B12</t>
+          <t>B8–B10</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>151 (chỉ có max+1)</t>
         </is>
       </c>
     </row>
     <row r="52" ht="62" customHeight="1">
       <c r="A52" s="6" t="inlineStr">
         <is>
+          <t>email — điều kiện ĐỊNH DẠNG</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>đúng định dạng email</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>sai định dạng
+null / rỗng</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>X8
+X10</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>(không áp dụng —
+miền rời rạc)</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>(không áp dụng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="62" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>6–30 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>&lt; 6 ký tự
 &gt; 30 ký tự
@@ -2479,7 +2520,7 @@
 null</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>X1
 X2
@@ -2487,49 +2528,65 @@
 X4</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>6, 7, 18, 29, 30</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>B14–B18</t>
         </is>
       </c>
-      <c r="H52" s="10" t="inlineStr">
+      <c r="H53" s="10" t="inlineStr">
         <is>
           <t>___________  ⟵ BẠN ĐIỀN</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="34" customHeight="1">
-      <c r="A54" s="11" t="inlineStr">
-        <is>
-          <t>GỢI Ý ô trống: khoảng hợp lệ của password là [6, 30]. Robustness BVA thêm đúng hai giá trị ngay NGOÀI biên — min−1 và max+1. Vậy hai số đó là gì? (xem lại dòng fullName và email ở trên để thấy quy luật).</t>
         </is>
       </c>
     </row>
     <row r="55" ht="34" customHeight="1">
       <c r="A55" s="11" t="inlineStr">
         <is>
-          <t>LƯU Ý QUAN TRỌNG khi thuyết trình: cột 'Valid Boundaries (Standard)' chỉ chứa giá trị HỢP LỆ — công thức 4n+1. Đối chiếu slide 29: khoảng [2, 64] cho ra 2, 3, 63, 64, 33; slide 31: khoảng [500, 9000] cho ra 500, 501, 4750, 8999, 9000. Không giá trị nào vượt ra ngoài khoảng. Giá trị ngoài biên thuộc cột Robustness (6n+1).</t>
+          <t>GỢI Ý ô trống: khoảng hợp lệ của password là [6, 30]. Robustness BVA thêm đúng hai giá trị ngay NGOÀI biên — min−1 và max+1. Vậy hai số đó là gì? (xem lại dòng fullName và email ở trên để thấy quy luật).</t>
         </is>
       </c>
     </row>
     <row r="56" ht="34" customHeight="1">
       <c r="A56" s="11" t="inlineStr">
         <is>
+          <t>LƯU Ý QUAN TRỌNG khi thuyết trình: cột 'Valid Boundaries (Standard)' chỉ chứa giá trị HỢP LỆ — công thức 4n+1. Đối chiếu slide 29: khoảng [2, 64] cho ra 2, 3, 63, 64, 33; slide 31: khoảng [500, 9000] cho ra 500, 501, 4750, 8999, 9000. Không giá trị nào vượt ra ngoài khoảng. Giá trị ngoài biên thuộc cột Robustness (6n+1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="34" customHeight="1">
+      <c r="A57" s="11" t="inlineStr">
+        <is>
+          <t>VÌ SAO EMAIL KHÔNG CÓ BIÊN DƯỚI: ràng buộc của email là @NotBlank + @Email + @Size(max = 150) — CHỈ khai max, không khai min. Đã kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều được chấp nhận. Vì thế Robustness của email chỉ có max+1 = 151, không có min−1. Khác với password (@Size khai min=6 nên min−1 = 5 là giá trị không hợp lệ thật) và fullName (biên dưới do @NotBlank sinh ra nên chuỗi rỗng chính là min−1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="34" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>VÌ SAO TÁCH EMAIL LÀM HAI DÒNG: theo mẫu slide 29, một trường có thể mang nhiều điều kiện độc lập — Customer name được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên; điều kiện ĐỊNH DẠNG là miền rời rạc (đúng/sai) nên chỉ phân lớp được, không có biên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="34" customHeight="1">
+      <c r="A59" s="11" t="inlineStr">
+        <is>
           <t>PHÁT HIỆN — lớp X3: chuỗi 8 dấu cách có độ dài 8 nên THOẢ MÃN @Size(min=6, max=30), nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên kỹ thuật giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện ra. Đây là bằng chứng hai kỹ thuật bổ sung cho nhau chứ không thay thế nhau.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="6">
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A54:H54"/>
     <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A58:H58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4190,12 +4247,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>$A$7:$A$46</t>
+          <t>$A$7:$A$47</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>40 case: 27 BVA + 13 EP</t>
+          <t>41 case: 28 BVA + 13 EP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(report): thống nhất thứ tự nhãn và đánh số B liên tục
Hai lỗi trong bảng thiết kế:
- Thứ tự hiển thị không khớp thứ tự nhãn: password mang V1 nhưng nằm cuối
  bảng, fullName mang V2 lại nằm đầu.
- Nhãn B nhảy số: B12 và B13 bị bỏ trống sau khi sửa lại phần email
  (email trước dùng B8-B13, sau khi bỏ min/min+1 chỉ còn B8-B11).

Sửa: thống nhất một chiều password (V1) -> fullName (V2) -> email (V3, V4)
cho cả danh sách case lẫn bảng thiết kế. Đánh lại nhãn B liên tục B1-B18:
  password B1-B5 (Standard) + B6, B7 (Robustness)
  fullName B8-B12 (Standard) + B13, B14 (Robustness)
  email    B15-B17 (Standard) + B18 (chỉ có max+1)

Thứ tự này khớp với tên hàm trong RegisterEquivalencePartitionTest
(V1/X1-X4 là password) nên đối chiếu code với báo cáo không lệch.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -150,11 +150,11 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -644,12 +644,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>fullName · Standard BVA</t>
+          <t>password · Standard BVA</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>min = 1 ký tự</t>
+          <t>min = 6 ký tự</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -686,12 +686,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>fullName · Standard BVA</t>
+          <t>password · Standard BVA</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>min+1 = 2 ký tự</t>
+          <t>min+1 = 7 ký tự</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -728,12 +728,12 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>fullName · Standard BVA</t>
+          <t>password · Standard BVA</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>nominal = 50 ký tự</t>
+          <t>nominal = 18 ký tự</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -770,12 +770,12 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>fullName · Standard BVA</t>
+          <t>password · Standard BVA</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>max-1 = 99 ký tự</t>
+          <t>max-1 = 29 ký tự</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>fullName · Standard BVA</t>
+          <t>password · Standard BVA</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>max = 100 ký tự</t>
+          <t>max = 30 ký tự</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -854,17 +854,17 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>fullName · Robustness / Negative</t>
+          <t>password · Robustness BVA</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>min-1 = rỗng</t>
+          <t>min-1 = 5 ký tự</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -896,17 +896,17 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>fullName · Robustness / Negative</t>
+          <t>password · Robustness BVA</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>blank = "   "</t>
+          <t>max+1 = 31 ký tự</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B7</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>fullName · Robustness / Negative</t>
+          <t>password · Negative</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -948,7 +948,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -980,17 +980,17 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>fullName · Robustness / Negative</t>
+          <t>password · Negative</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>max+1 = 101</t>
+          <t>empty = rỗng</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -1005,7 +1005,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>B7</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA (chỉ có biên trên)</t>
+          <t>fullName · Standard BVA</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>giá trị ngắn hợp lệ (không phải biên) = 6 ký tự</t>
+          <t>min = 1 ký tự</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="H16" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B8</t>
         </is>
       </c>
     </row>
@@ -1064,12 +1064,12 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>email · Standard BVA (chỉ có biên trên)</t>
+          <t>fullName · Standard BVA</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>giá trị ngắn hợp lệ (không phải biên) = 7 ký tự</t>
+          <t>min+1 = 2 ký tự</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B9</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA (chỉ có biên trên)</t>
+          <t>fullName · Standard BVA</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>nominal = 75 ký tự</t>
+          <t>nominal = 50 ký tự</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="H18" s="8" t="inlineStr">
         <is>
-          <t>B8</t>
+          <t>B10</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>email · Standard BVA (chỉ có biên trên)</t>
+          <t>fullName · Standard BVA</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>max-1 = 149 ký tự</t>
+          <t>max-1 = 99 ký tự</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>B9</t>
+          <t>B11</t>
         </is>
       </c>
     </row>
@@ -1190,12 +1190,12 @@
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>email · Standard BVA (chỉ có biên trên)</t>
+          <t>fullName · Standard BVA</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>max = 150 ký tự</t>
+          <t>max = 100 ký tự</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H20" s="8" t="inlineStr">
         <is>
-          <t>B10</t>
+          <t>B12</t>
         </is>
       </c>
     </row>
@@ -1232,17 +1232,17 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>email · Robustness</t>
+          <t>fullName · Robustness BVA</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>max+1 = 151 ký tự</t>
+          <t>min-1 = rỗng (0 ký tự)</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Size)</t>
+          <t>Bị từ chối</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>B11</t>
+          <t>B13</t>
         </is>
       </c>
     </row>
@@ -1274,17 +1274,17 @@
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>email · Negative (điều kiện định dạng)</t>
+          <t>fullName · Robustness BVA</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>null = null</t>
+          <t>max+1 = 101 ký tự</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Email / @NotBlank)</t>
+          <t>Bị từ chối</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="H22" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>B14</t>
         </is>
       </c>
     </row>
@@ -1316,17 +1316,17 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>email · Negative (điều kiện định dạng)</t>
+          <t>fullName · Negative</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>empty = rỗng</t>
+          <t>blank = toàn khoảng trắng</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Email / @NotBlank)</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1358,17 +1358,17 @@
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>email · Negative (điều kiện định dạng)</t>
+          <t>fullName · Negative</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>invalid format = sai định dạng</t>
+          <t>null = null</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Email / @NotBlank)</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H24" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1400,12 +1400,12 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>password · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>min = 6 ký tự</t>
+          <t>giá trị ngắn hợp lệ (không phải biên) = 6 ký tự</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>B14</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1442,12 +1442,12 @@
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>password · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>min+1 = 7 ký tự</t>
+          <t>giá trị ngắn hợp lệ (không phải biên) = 7 ký tự</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="H26" s="8" t="inlineStr">
         <is>
-          <t>B15</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1484,12 +1484,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>password · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>nominal = 18 ký tự</t>
+          <t>nominal = 75 ký tự</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -1509,7 +1509,7 @@
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>B16</t>
+          <t>B15</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
-          <t>password · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
         <is>
-          <t>max-1 = 29 ký tự</t>
+          <t>max-1 = 149 ký tự</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="H28" s="8" t="inlineStr">
         <is>
-          <t>B17</t>
+          <t>B16</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1568,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>password · Standard BVA</t>
+          <t>email · Standard BVA (chỉ có biên trên)</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>max = 30 ký tự</t>
+          <t>max = 150 ký tự</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>B18</t>
+          <t>B17</t>
         </is>
       </c>
     </row>
@@ -1610,17 +1610,17 @@
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>password · Robustness / Negative</t>
+          <t>email · Robustness BVA</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
         <is>
-          <t>min-1 = 5</t>
+          <t>max+1 = 151 ký tự</t>
         </is>
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="H30" s="8" t="inlineStr">
         <is>
-          <t>B19</t>
+          <t>B18</t>
         </is>
       </c>
     </row>
@@ -1652,17 +1652,17 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>password · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>max+1 = 31</t>
+          <t>null = null</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>B20</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1694,17 +1694,17 @@
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>password · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D32" s="8" t="inlineStr">
         <is>
-          <t>null = null</t>
+          <t>empty = rỗng</t>
         </is>
       </c>
       <c r="E32" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F32" s="8" t="inlineStr">
@@ -1719,7 +1719,7 @@
       </c>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -1736,17 +1736,17 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>password · Robustness / Negative</t>
+          <t>email · Negative (điều kiện định dạng)</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>empty = rỗng</t>
+          <t>invalid format = sai định dạng</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối</t>
+          <t>Bị từ chối (@Email / @NotBlank)</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>–</t>
         </is>
       </c>
     </row>
@@ -2363,156 +2363,21 @@
     <row r="50" ht="62" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>fullName</t>
+          <t>password</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
-        <is>
-          <t>1–100 ký tự,
-có ít nhất 1 ký tự không trắng</t>
-        </is>
-      </c>
-      <c r="C50" s="6" t="inlineStr">
-        <is>
-          <t>V2</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>rỗng / toàn khoảng trắng
-&gt; 100 ký tự
-null</t>
-        </is>
-      </c>
-      <c r="E50" s="6" t="inlineStr">
-        <is>
-          <t>X6
-X5
-X7</t>
-        </is>
-      </c>
-      <c r="F50" s="6" t="inlineStr">
-        <is>
-          <t>1, 2, 50, 99, 100</t>
-        </is>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>B1–B5</t>
-        </is>
-      </c>
-      <c r="H50" s="6" t="inlineStr">
-        <is>
-          <t>rỗng (= min−1), 101</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="62" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>email — điều kiện ĐỘ DÀI</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>≤ 150 ký tự</t>
-        </is>
-      </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t>V3</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>&gt; 150 ký tự</t>
-        </is>
-      </c>
-      <c r="E51" s="6" t="inlineStr">
-        <is>
-          <t>X9</t>
-        </is>
-      </c>
-      <c r="F51" s="6" t="inlineStr">
-        <is>
-          <t>75, 149, 150
-(không có biên dưới)</t>
-        </is>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>B8–B10</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
-        <is>
-          <t>151 (chỉ có max+1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="62" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
-        <is>
-          <t>email — điều kiện ĐỊNH DẠNG</t>
-        </is>
-      </c>
-      <c r="B52" s="6" t="inlineStr">
-        <is>
-          <t>đúng định dạng email</t>
-        </is>
-      </c>
-      <c r="C52" s="6" t="inlineStr">
-        <is>
-          <t>V4</t>
-        </is>
-      </c>
-      <c r="D52" s="6" t="inlineStr">
-        <is>
-          <t>sai định dạng
-null / rỗng</t>
-        </is>
-      </c>
-      <c r="E52" s="6" t="inlineStr">
-        <is>
-          <t>X8
-X10</t>
-        </is>
-      </c>
-      <c r="F52" s="6" t="inlineStr">
-        <is>
-          <t>(không áp dụng —
-miền rời rạc)</t>
-        </is>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H52" s="6" t="inlineStr">
-        <is>
-          <t>(không áp dụng)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="62" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
-        <is>
-          <t>password</t>
-        </is>
-      </c>
-      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>6–30 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C50" s="6" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D50" s="6" t="inlineStr">
         <is>
           <t>&lt; 6 ký tự
 &gt; 30 ký tự
@@ -2520,7 +2385,7 @@
 null</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E50" s="6" t="inlineStr">
         <is>
           <t>X1
 X2
@@ -2528,52 +2393,190 @@
 X4</t>
         </is>
       </c>
+      <c r="F50" s="6" t="inlineStr">
+        <is>
+          <t>6, 7, 18, 29, 30</t>
+        </is>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>B1–B5</t>
+        </is>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
+        <is>
+          <t>5 và 31
+(B6, B7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="62" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>fullName</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>1–100 ký tự,
+có ít nhất 1 ký tự không trắng</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>V2</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 100 ký tự
+toàn khoảng trắng
+null</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>X5
+X6
+X7</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>1, 2, 50, 99, 100</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>B8–B12</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>rỗng (= min−1) và 101
+(B13, B14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="62" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>email — điều kiện ĐỘ DÀI</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>≤ 150 ký tự</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 150 ký tự</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>X9</t>
+        </is>
+      </c>
+      <c r="F52" s="6" t="inlineStr">
+        <is>
+          <t>75, 149, 150
+(KHÔNG có biên dưới)</t>
+        </is>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>B15–B17</t>
+        </is>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
+        <is>
+          <t>151
+(B18, chỉ có max+1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="62" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>email — điều kiện ĐỊNH DẠNG</t>
+        </is>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>đúng định dạng email</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>V4</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>sai định dạng
+null / rỗng</t>
+        </is>
+      </c>
+      <c r="E53" s="6" t="inlineStr">
+        <is>
+          <t>X8
+X10</t>
+        </is>
+      </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>6, 7, 18, 29, 30</t>
+          <t>(không áp dụng —
+miền rời rạc)</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>B14–B18</t>
-        </is>
-      </c>
-      <c r="H53" s="10" t="inlineStr">
-        <is>
-          <t>___________  ⟵ BẠN ĐIỀN</t>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>(không áp dụng)</t>
         </is>
       </c>
     </row>
     <row r="55" ht="34" customHeight="1">
-      <c r="A55" s="11" t="inlineStr">
+      <c r="A55" s="10" t="inlineStr">
         <is>
           <t>GỢI Ý ô trống: khoảng hợp lệ của password là [6, 30]. Robustness BVA thêm đúng hai giá trị ngay NGOÀI biên — min−1 và max+1. Vậy hai số đó là gì? (xem lại dòng fullName và email ở trên để thấy quy luật).</t>
         </is>
       </c>
     </row>
     <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
+      <c r="A56" s="10" t="inlineStr">
         <is>
           <t>LƯU Ý QUAN TRỌNG khi thuyết trình: cột 'Valid Boundaries (Standard)' chỉ chứa giá trị HỢP LỆ — công thức 4n+1. Đối chiếu slide 29: khoảng [2, 64] cho ra 2, 3, 63, 64, 33; slide 31: khoảng [500, 9000] cho ra 500, 501, 4750, 8999, 9000. Không giá trị nào vượt ra ngoài khoảng. Giá trị ngoài biên thuộc cột Robustness (6n+1).</t>
         </is>
       </c>
     </row>
     <row r="57" ht="34" customHeight="1">
-      <c r="A57" s="11" t="inlineStr">
+      <c r="A57" s="10" t="inlineStr">
         <is>
           <t>VÌ SAO EMAIL KHÔNG CÓ BIÊN DƯỚI: ràng buộc của email là @NotBlank + @Email + @Size(max = 150) — CHỈ khai max, không khai min. Đã kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều được chấp nhận. Vì thế Robustness của email chỉ có max+1 = 151, không có min−1. Khác với password (@Size khai min=6 nên min−1 = 5 là giá trị không hợp lệ thật) và fullName (biên dưới do @NotBlank sinh ra nên chuỗi rỗng chính là min−1).</t>
         </is>
       </c>
     </row>
     <row r="58" ht="34" customHeight="1">
-      <c r="A58" s="11" t="inlineStr">
+      <c r="A58" s="10" t="inlineStr">
         <is>
           <t>VÌ SAO TÁCH EMAIL LÀM HAI DÒNG: theo mẫu slide 29, một trường có thể mang nhiều điều kiện độc lập — Customer name được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên; điều kiện ĐỊNH DẠNG là miền rời rạc (đúng/sai) nên chỉ phân lớp được, không có biên.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="11" t="inlineStr">
+      <c r="A59" s="10" t="inlineStr">
         <is>
           <t>PHÁT HIỆN — lớp X3: chuỗi 8 dấu cách có độ dài 8 nên THOẢ MÃN @Size(min=6, max=30), nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên kỹ thuật giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện ra. Đây là bằng chứng hai kỹ thuật bổ sung cho nhau chứ không thay thế nhau.</t>
         </is>
@@ -3167,7 +3170,7 @@
       <c r="H19" s="6" t="inlineStr"/>
     </row>
     <row r="21" ht="34" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Số rule tối đa = tích số giá trị các điều kiện = 3 × 2 = 6. Đây là tiêu chí ĐỦ của kỹ thuật: phủ hết 6 rule thì chứng minh được không sót tổ hợp nào.</t>
         </is>
@@ -3324,14 +3327,14 @@
           <t>Vì sao gộp được R1 và R2?</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>_______________________________________________  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
     </row>
     <row r="31" ht="34" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>GỢI Ý: nhìn R1 và R2 ở bảng đầy đủ — cùng C1 = NOT_STARTED nhưng C2 khác nhau, mà kết quả A1/A2 lại GIỐNG HỆT. Khi kết quả không đổi dù điều kiện đổi, nghĩa là điều kiện đó không ảnh hưởng, ta điền dấu '–' và gộp hai cột làm một. Slide 46 có ví dụ y hệt với bài toán thuế.</t>
         </is>
@@ -4116,17 +4119,17 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
-      <c r="C26" s="10" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
@@ -4136,7 +4139,7 @@
           <t>KHÔNG</t>
         </is>
       </c>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
@@ -4145,14 +4148,14 @@
       <c r="H26" s="6" t="inlineStr"/>
     </row>
     <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>TIÊU CHÍ ĐỦ của kỹ thuật này: phủ hết CẠNH của sơ đồ. Ba trạng thái sinh ra 3 × 2 = 6 cặp có thứ tự, tức 6 cạnh. Dòng 1–6 phủ đủ 6 cạnh đó. Dòng 7–8 là chuyển đổi bị chặn.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>GỢI Ý dòng 9: còn MỘT trạng thái đầu nữa chưa được thử với node bị khoá. Nhìn cột Start State của dòng 7 và 8 — thiếu trạng thái nào trong ba trạng thái?</t>
         </is>
@@ -4164,14 +4167,14 @@
           <t>SƠ ĐỒ TRẠNG THÁI</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>[ CHÈN ẢNH SƠ ĐỒ BẠN VẼ VÀO ĐÂY ]  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
     </row>
     <row r="32" ht="34" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Sơ đồ cần: 3 ô trạng thái, 6 mũi tên chuyển, và ghi chú mũi tên nào bị chặn khi node khoá. Vẽ tay chụp ảnh cũng được.</t>
         </is>
@@ -4301,7 +4304,7 @@
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Cách gộp: chuột phải tab sheet → Move or Copy → chọn file All_Methods → tick 'Create a copy'. Sau đó mở sheet '00. Tổng quan' của file All_Methods, sửa lại vùng trong công thức COUNTA/COUNTIF cho khớp cột 'Vùng công thức A4' ở trên.</t>
         </is>

</xml_diff>

<commit_message>
docs(report): EP-10 phủ cả V3 và V4, bổ sung quy tắc gộp lớp hợp lệ
Nhãn của EP-10 chỉ ghi V3 khiến V4 (lớp định dạng email hợp lệ) trông như
chưa được phủ. Thực tế giá trị "sinhvien@uth.edu.vn" thoả cả hai lớp cùng
lúc: độ dài 19 <= 150 (V3) và đúng định dạng (V4). Sửa nhãn thành V3 + V4.

Bổ sung ghi chú giải thích quy tắc của kỹ thuật:
- Lớp HỢP LỆ gộp được, một test phủ nhiều lớp V cùng lúc.
- Lớp KHÔNG hợp lệ phải tách riêng, vì nếu một test vi phạm hai ràng buộc
  thì ràng buộc bắt trước sẽ che mất ràng buộc kia (masking), không biết
  cái còn lại có được kiểm hay không.
- Đây cũng là lý do dùng validateProperty(dto, field) thay vì validate(dto).

Kiểm chứng độ phủ: V1-V4 đủ 4/4, X1-X10 đủ 10/10, nhãn B1-B18 liên tục.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2161,7 +2161,7 @@
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>V3 — "sinhvien@uth.edu.vn"</t>
+          <t>V3 + V4 — "sinhvien@uth.edu.vn"</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>v3_email_lopHopLe</t>
+          <t>Một test phủ CẢ HAI lớp hợp lệ: độ dài (V3) và định dạng (V4)</t>
         </is>
       </c>
     </row>
@@ -2564,31 +2564,39 @@
     <row r="57" ht="34" customHeight="1">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>VÌ SAO EMAIL KHÔNG CÓ BIÊN DƯỚI: ràng buộc của email là @NotBlank + @Email + @Size(max = 150) — CHỈ khai max, không khai min. Đã kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều được chấp nhận. Vì thế Robustness của email chỉ có max+1 = 151, không có min−1. Khác với password (@Size khai min=6 nên min−1 = 5 là giá trị không hợp lệ thật) và fullName (biên dưới do @NotBlank sinh ra nên chuỗi rỗng chính là min−1).</t>
+          <t>QUY TẮC GỘP LỚP HỢP LỆ: một test case có thể phủ NHIỀU lớp hợp lệ cùng lúc — EP-10 dùng "sinhvien@uth.edu.vn" vừa thoả V3 (độ dài ≤ 150) vừa thoả V4 (đúng định dạng), nên phủ luôn cả hai. Ngược lại, lớp KHÔNG hợp lệ phải tách riêng từng test: nếu một test vừa sai định dạng vừa quá 150 ký tự thì ràng buộc nào bắt trước sẽ CHE MẤT ràng buộc kia, không biết cái còn lại có được kiểm hay không. Đây cũng là lý do bạn Quân dùng validateProperty(dto, "password") thay vì validate(dto) — để cô lập đúng một trường.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="34" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>VÌ SAO TÁCH EMAIL LÀM HAI DÒNG: theo mẫu slide 29, một trường có thể mang nhiều điều kiện độc lập — Customer name được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên; điều kiện ĐỊNH DẠNG là miền rời rạc (đúng/sai) nên chỉ phân lớp được, không có biên.</t>
+          <t>VÌ SAO EMAIL KHÔNG CÓ BIÊN DƯỚI: ràng buộc của email là @NotBlank + @Email + @Size(max = 150) — CHỈ khai max, không khai min. Đã kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều được chấp nhận. Vì thế Robustness của email chỉ có max+1 = 151, không có min−1. Khác với password (@Size khai min=6 nên min−1 = 5 là giá trị không hợp lệ thật) và fullName (biên dưới do @NotBlank sinh ra nên chuỗi rỗng chính là min−1).</t>
         </is>
       </c>
     </row>
     <row r="59" ht="34" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
+          <t>VÌ SAO TÁCH EMAIL LÀM HAI DÒNG: theo mẫu slide 29, một trường có thể mang nhiều điều kiện độc lập — Customer name được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên; điều kiện ĐỊNH DẠNG là miền rời rạc (đúng/sai) nên chỉ phân lớp được, không có biên.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="34" customHeight="1">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
           <t>PHÁT HIỆN — lớp X3: chuỗi 8 dấu cách có độ dài 8 nên THOẢ MÃN @Size(min=6, max=30), nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên kỹ thuật giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện ra. Đây là bằng chứng hai kỹ thuật bổ sung cho nhau chứ không thay thế nhau.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A55:H55"/>
     <mergeCell ref="A59:H59"/>
     <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A60:H60"/>
     <mergeCell ref="A58:H58"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(blackbox): bảng quyết định thứ hai - hiệu lực token đặt lại mật khẩu
PasswordResetToken.isValid() = !isExpired() && !isUsed() — hai điều kiện nhị
phân độc lập, số rule tối đa 2 x 2 = 4. Bảng này bổ sung cho bảng
ProgressService (3 x 2 = 6) và cho thấy công thức 2^n chỉ đúng khi MỌI điều
kiện đều nhị phân.

Phát hiện: PasswordResetServiceTest sẵn có chỉ phủ R1 và R2 cho validateToken.
R3 (còn hạn nhưng đã dùng) chỉ được chạm gián tiếp qua resetPassword - một
phương thức khác. R4 (vừa hết hạn vừa đã dùng) chưa từng được test.

Thêm sheet 03b vào báo cáo với bảng đầy đủ 4 rule và bản rút gọn còn 3 cột,
kèm sắp lại thứ tự sheet cho đúng mạch đọc.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01. BVA + Equiv Partition" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03. Decision Table (PhanA)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04. State Transition (PhanA)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99. Huong dan gop" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03b. Decision Table Token" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04. State Transition (PhanA)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99. Huong dan gop" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3365,6 +3366,646 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Decision Table Testing — bảng thứ hai</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Hiệu lực token đặt lại mật khẩu: PasswordResetToken.isValid(). Bảng thiết kế theo mẫu slide 44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tổng case</t>
+        </is>
+      </c>
+      <c r="B4" s="4">
+        <f>COUNTA($A$7:$A$10)</f>
+        <v/>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="D4" s="4">
+        <f>COUNTIF($G$7:$G$10,"PASS")</f>
+        <v/>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Chưa chạy</t>
+        </is>
+      </c>
+      <c r="F4" s="4">
+        <f>COUNTIF($G$7:$G$10,"Chưa chạy")</f>
+        <v/>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Known bug</t>
+        </is>
+      </c>
+      <c r="H4" s="4">
+        <f>COUNTIF($G$7:$G$10,"KNOWN BUG")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Case ID</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Source test</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Test category</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Input / condition</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Expected result</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Actual / evidence</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>DT-B01</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>TokenValidityDecisionTableTest</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>C1=còn hạn; C2=chưa dùng</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Token vừa tạo, chưa ai dùng</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Token HỢP LỆ</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>R1 · rule1_conHan_chuaDung_hopLe</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DT-B02</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>TokenValidityDecisionTableTest</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>C1=hết hạn; C2=chưa dùng</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Quá 30 phút, chưa ai dùng</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>Token không hợp lệ</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>R2 · rule2_hetHan_chuaDung_khongHopLe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>DT-B03</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>TokenValidityDecisionTableTest</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>C1=còn hạn; C2=đã dùng</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Còn hạn nhưng đã đặt lại mật khẩu rồi</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Token không hợp lệ</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>R3 · trước đây chỉ chạm gián tiếp qua resetPassword</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>DT-B04</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>TokenValidityDecisionTableTest</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>C1=hết hạn; C2=đã dùng</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Vừa quá hạn vừa đã dùng</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Token không hợp lệ</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>R4 · TỔ HỢP TRƯỚC ĐÂY CHƯA TỪNG TEST</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>BẢNG QUYẾT ĐỊNH ĐẦY ĐỦ — mẫu slide 44</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Condition / Action</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>R3</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>R4</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>C1 · Token đã hết hạn</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>2 giá trị</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>C2 · Token đã được dùng</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>2 giá trị</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>A1 · Token HỢP LỆ</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr"/>
+      <c r="H16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>A2 · Token KHÔNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Số rule tối đa = 2 × 2 = 4. Ở bảng này CẢ HAI điều kiện đều nhị phân nên công thức 2^n áp dụng được. Khác với bảng ProgressService (3 × 2 = 6) nơi điều kiện trạng thái có ba giá trị — lúc đó phải NHÂN chứ không luỹ thừa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>BẢNG SAU KHI RÚT GỌN — bước 6 slide 42</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Condition / Action</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>R1'</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>R2'</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>R3'</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>C1 · Token đã hết hạn</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
+      <c r="F22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr"/>
+      <c r="H22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>C2 · Token đã được dùng</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr"/>
+      <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr"/>
+      <c r="H23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>A1 · Token HỢP LỆ</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr"/>
+      <c r="H24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>A2 · Token KHÔNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
+      <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr"/>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>gộp R2, R3, R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Vì sao ba rule R2, R3, R4 gộp được?</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>_______________________________________________  ⟵ BẠN ĐIỀN</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>GỢI Ý: nhìn công thức isValid() = !isExpired() &amp;&amp; !isUsed(). Với phép AND, chỉ cần MỘT vế sai là cả biểu thức sai. Vậy khi token đã hết hạn thì việc nó đã dùng hay chưa có làm thay đổi kết quả không? Điều kiện không ảnh hưởng thì điền dấu '–'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>PHÁT HIỆN: PasswordResetServiceTest sẵn có chỉ phủ R1 và R2 cho validateToken. Rule R3 (còn hạn nhưng đã dùng) chỉ được chạm gián tiếp qua resetPassword — một phương thức khác. Rule R4 (vừa hết hạn vừa đã dùng) chưa từng được test. Lập bảng đầy đủ 4 rule mới thấy hai lỗ hổng này.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A12:H12"/>
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A19:H19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4199,13 +4840,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4285,113 +4926,135 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>6 case, phủ đủ 6 rule</t>
+          <t>6 case, phủ đủ 6 rule (3 × 2)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
+          <t>03b. Decision Table Token</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Thêm mới, đặt cạnh sheet 03</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>$A$7:$A$10</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>4 case, phủ đủ 4 rule (2 × 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
           <t>04. State Transition (PhanA)</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Thay cho '04. State Transition'</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>$A$7:$A$14</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>8 case, phủ đủ 6 cạnh + 2 chặn</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Cách gộp: chuột phải tab sheet → Move or Copy → chọn file All_Methods → tick 'Create a copy'. Sau đó mở sheet '00. Tổng quan' của file All_Methods, sửa lại vùng trong công thức COUNTA/COUNTIF cho khớp cột 'Vùng công thức A4' ở trên.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>KHÁC BIỆT SO VỚI BẢN CŨ CỦA NHÓM</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Bản cũ</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Bản này</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>Cột bằng chứng ghi 'Unit test hiện có' — gán ngược test có sẵn vào tên kỹ thuật</t>
+          <t>Bản cũ</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Mỗi hàm test đặt tên theo mã dòng bảng thiết kế (rule3_, st05_) — thiết kế trước, code sau</t>
+          <t>Bản này</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>Không có bảng thiết kế theo mẫu slide</t>
+          <t>Cột bằng chứng ghi 'Unit test hiện có' — gán ngược test có sẵn vào tên kỹ thuật</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Có bảng slide 32 (phân lớp + biên), slide 44 (quyết định), slide 39 (chuyển trạng thái)</t>
+          <t>Mỗi hàm test đặt tên theo mã dòng bảng thiết kế (rule3_, st05_) — thiết kế trước, code sau</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>Decision Table: 4 tổ hợp, trong đó 1 dòng khai sai độ phủ</t>
+          <t>Không có bảng thiết kế theo mẫu slide</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>6 tổ hợp — đủ 3 × 2, phát hiện tổ hợp IN_PROGRESS + khoá trước đây chưa có test</t>
+          <t>Có bảng slide 32 (phân lớp + biên), slide 44 (quyết định), slide 39 (chuyển trạng thái)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>State Transition: chỉ chuyển đổi hợp lệ</t>
+          <t>Decision Table: 4 tổ hợp, trong đó 1 dòng khai sai độ phủ</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Đủ 6 cạnh + 2 chuyển đổi bị chặn</t>
+          <t>6 tổ hợp — đủ 3 × 2, phát hiện tổ hợp IN_PROGRESS + khoá trước đây chưa có test</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t>State Transition: chỉ chuyển đổi hợp lệ</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Đủ 6 cạnh + 2 chuyển đổi bị chặn</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t>Equivalence Partitioning: suy ra từ BVA</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>13 case độc lập, phát hiện lớp 'toàn khoảng trắng' mà BVA không chạm tới</t>
         </is>
@@ -4399,8 +5062,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A9:F9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(report): bảng rút gọn không chồng lấn + ghi lý do rút gọn
Bảng rút gọn của sheet 03b có R3' = (C1=–, C2=Y) khiến tổ hợp (Y, Y) khớp
cả R2' lẫn R3' — rule R4 bị phủ hai lần. Không sai kết quả vì cả hai đều cho
A2, nhưng bảng quyết định chuẩn nên để mỗi bộ đầu vào khớp đúng một cột.
Sửa R3' thành (C1=N, C2=Y): ba cột phủ gọn 4 rule là (N,N), (Y,*), (N,Y).

Ghi lý do rút gọn của cả hai bảng vào báo cáo, kèm nguyên nhân ở tầng mã
nguồn: phép && bị đoản mạch nên điều kiện thứ hai không được đánh giá.
Bảng 03 có bằng chứng trực tiếp trong test:
verify(roadmapService, never()).isNodeLocked(...).
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -91,12 +91,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -155,10 +155,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3336,9 +3336,9 @@
           <t>Vì sao gộp được R1 và R2?</t>
         </is>
       </c>
-      <c r="B29" s="11" t="inlineStr">
-        <is>
-          <t>_______________________________________________  ⟵ BẠN ĐIỀN</t>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Vì R1 và R2 cho thấy việc C2 không ảnh hưởng đến Action, nên có thể rút gọn thành "–". Nguyên nhân sâu hơn: phép &amp;&amp; trong !NOT_STARTED.equals(status) &amp;&amp; isNodeLocked(...) bị đoản mạch — khi trạng thái là NOT_STARTED thì vế đầu đã sai, Java không gọi isNodeLocked() nữa. Test kiểm chứng bằng verify(roadmapService, never()).isNodeLocked(...).</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
@@ -3968,33 +3968,41 @@
           <t>Vì sao ba rule R2, R3, R4 gộp được?</t>
         </is>
       </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>_______________________________________________  ⟵ BẠN ĐIỀN</t>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>R2 và R4 cho thấy C2 không ảnh hưởng đến kết quả khi token đã hết hạn → gộp thành R2' (C1=Y, C2=–). R3 giữ nguyên thành R3' (C1=N, C2=Y). Nguyên nhân: isValid() = !isExpired() &amp;&amp; !isUsed(), phép &amp;&amp; chỉ cần MỘT vế sai là cả biểu thức sai, nên hết hạn HOẶC đã dùng đều cho ra không hợp lệ.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>GỢI Ý: nhìn công thức isValid() = !isExpired() &amp;&amp; !isUsed(). Với phép AND, chỉ cần MỘT vế sai là cả biểu thức sai. Vậy khi token đã hết hạn thì việc nó đã dùng hay chưa có làm thay đổi kết quả không? Điều kiện không ảnh hưởng thì điền dấu '–'.</t>
+          <t>LƯU Ý VỀ CHẤT LƯỢNG RÚT GỌN: bảng rút gọn nên có các rule KHÔNG CHỒNG LẤN — mỗi bộ đầu vào chỉ khớp đúng một cột. Nếu đặt R3' là (C1=–, C2=Y) thì tổ hợp (Y, Y) sẽ khớp cả R2' lẫn R3', tức R4 bị đếm hai lần. Đặt R3' là (C1=N, C2=Y) thì ba cột phủ gọn 4 rule: (N,N), (Y,*), (N,Y) — không cột nào giẫm lên cột nào.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="34" customHeight="1">
       <c r="A30" s="10" t="inlineStr">
         <is>
+          <t>GỢI Ý: nhìn công thức isValid() = !isExpired() &amp;&amp; !isUsed(). Với phép AND, chỉ cần MỘT vế sai là cả biểu thức sai. Vậy khi token đã hết hạn thì việc nó đã dùng hay chưa có làm thay đổi kết quả không? Điều kiện không ảnh hưởng thì điền dấu '–'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
           <t>PHÁT HIỆN: PasswordResetServiceTest sẵn có chỉ phủ R1 và R2 cho validateToken. Rule R3 (còn hạn nhưng đã dùng) chỉ được chạm gián tiếp qua resetPassword — một phương thức khác. Rule R4 (vừa hết hạn vừa đã dùng) chưa từng được test. Lập bảng đầy đủ 4 rule mới thấy hai lỗ hổng này.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4715,7 +4723,7 @@
           <t>Bị chặn (403)</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>KHÔNG</t>
         </is>
@@ -4749,7 +4757,7 @@
           <t>Bị chặn (403)</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>KHÔNG</t>
         </is>
@@ -4768,27 +4776,27 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="12" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
-      <c r="D26" s="11" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>KHÔNG</t>
         </is>
       </c>
-      <c r="F26" s="11" t="inlineStr">
+      <c r="F26" s="12" t="inlineStr">
         <is>
           <t>___  ⟵ BẠN ĐIỀN</t>
         </is>
@@ -4816,7 +4824,7 @@
           <t>SƠ ĐỒ TRẠNG THÁI</t>
         </is>
       </c>
-      <c r="B30" s="11" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>[ CHÈN ẢNH SƠ ĐỒ BẠN VẼ VÀO ĐÂY ]  ⟵ BẠN ĐIỀN</t>
         </is>

</xml_diff>

<commit_message>
docs(report): giữ quy ước rút gọn tối giản logic, trả lại lời văn của người thực hiện
Đổi R3' về (C1 = –, C2 = Y) theo hướng tối giản logic: dấu – đặt ở mọi điều
kiện không ảnh hưởng kết quả. Hệ quả là tổ hợp (Y, Y) khớp cả R2' lẫn R3',
nhưng không sai vì hai cột cùng dẫn tới hành động A2.

Ghi chú dưới bảng nêu rõ đây là lựa chọn có chủ đích và nêu phương án thay
thế (R3' = (N, Y)) nếu muốn các rule không chồng lấn.

Phần trả lời 'vì sao rút gọn được' giữ nguyên văn của người thực hiện; phần
giải thích sâu hơn (đoản mạch &&) tách thành ghi chú riêng bên dưới.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -3338,7 +3338,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Vì R1 và R2 cho thấy việc C2 không ảnh hưởng đến Action, nên có thể rút gọn thành "–". Nguyên nhân sâu hơn: phép &amp;&amp; trong !NOT_STARTED.equals(status) &amp;&amp; isNodeLocked(...) bị đoản mạch — khi trạng thái là NOT_STARTED thì vế đầu đã sai, Java không gọi isNodeLocked() nữa. Test kiểm chứng bằng verify(roadmapService, never()).isNodeLocked(...).</t>
+          <t>Vì R1 và R2 cho thấy việc C2 không ảnh hưởng đến Action, nên có thể rút gọn thành "–"</t>
         </is>
       </c>
     </row>
@@ -3872,7 +3872,7 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>–</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr"/>
@@ -3970,14 +3970,15 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>R2 và R4 cho thấy C2 không ảnh hưởng đến kết quả khi token đã hết hạn → gộp thành R2' (C1=Y, C2=–). R3 giữ nguyên thành R3' (C1=N, C2=Y). Nguyên nhân: isValid() = !isExpired() &amp;&amp; !isUsed(), phép &amp;&amp; chỉ cần MỘT vế sai là cả biểu thức sai, nên hết hạn HOẶC đã dùng đều cho ra không hợp lệ.</t>
+          <t>R2 - R4 cho thấy C2 không ảnh hưởng đến kết quả =&gt; Rút gọn thành R2'
+R3 - R4 cho thấy C1 không ảnh hưởng đến kết quả =&gt; Rút gọn thành R3'</t>
         </is>
       </c>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>LƯU Ý VỀ CHẤT LƯỢNG RÚT GỌN: bảng rút gọn nên có các rule KHÔNG CHỒNG LẤN — mỗi bộ đầu vào chỉ khớp đúng một cột. Nếu đặt R3' là (C1=–, C2=Y) thì tổ hợp (Y, Y) sẽ khớp cả R2' lẫn R3', tức R4 bị đếm hai lần. Đặt R3' là (C1=N, C2=Y) thì ba cột phủ gọn 4 rule: (N,N), (Y,*), (N,Y) — không cột nào giẫm lên cột nào.</t>
+          <t>QUY ƯỚC RÚT GỌN DÙNG Ở ĐÂY: bảng theo hướng tối giản logic — dấu '–' đặt ở mọi điều kiện không ảnh hưởng tới kết quả. Hệ quả: tổ hợp (hết hạn = Y, đã dùng = Y) khớp cả R2' lẫn R3'. Điều này KHÔNG sai vì cả hai cột đều dẫn tới cùng hành động A2, chỉ là một tổ hợp được phủ bởi hai cột. Nếu muốn mỗi tổ hợp chỉ khớp đúng một cột thì đổi R3' thành (C1 = N, C2 = Y) — cũng ba cột, cũng phủ đủ 4 rule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(report): nhóm bảng chuyển trạng thái theo Start State + sơ đồ draw.io
Bảng cũ liệt kê lộn xộn theo thứ tự viết test, khó theo dõi. Nhóm lại theo
trạng thái xuất phát, mỗi nhóm đúng 3 dòng: 2 chuyển đổi hợp lệ + 1 chuyển
đổi bị chặn khi node khoá.
  NOT_STARTED  dòng 1-3
  IN_PROGRESS  dòng 4-6
  DONE         dòng 7-9 (dòng 9 để trống cho người thực hiện tự điền)

Thêm SoDo-ChuyenTrangThai.drawio: 3 trạng thái, đủ 6 cạnh chuyển, phân biệt
bằng màu - đỏ nét đứt là chuyển đổi bị chặn khi node khoá (đi vào IN_PROGRESS
hoặc DONE), xanh nét liền là luôn được phép (đi vào NOT_STARTED). Có chú giải
và trích luật chặn từ mã nguồn.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -4135,12 +4135,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>NOT_STARTED · hợp lệ</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED + đánh dấu IN_PROGRESS</t>
+          <t>Đánh dấu IN_PROGRESS, node mở khoá</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -4177,12 +4177,12 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>NOT_STARTED · hợp lệ</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>IN_PROGRESS + đánh dấu DONE</t>
+          <t>Đánh dấu DONE, node mở khoá (nhảy cóc)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="H8" s="8" t="inlineStr">
         <is>
-          <t>st02</t>
+          <t>st05 · CẠNH BỔ SUNG</t>
         </is>
       </c>
     </row>
@@ -4219,17 +4219,17 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>NOT_STARTED · KHÔNG hợp lệ</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>DONE + bỏ đánh dấu</t>
+          <t>Đánh dấu DONE khi node BỊ KHOÁ</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED, xoá completedAt</t>
+          <t>Bị chặn 403, không lưu</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>st03</t>
+          <t>st07</t>
         </is>
       </c>
     </row>
@@ -4261,17 +4261,17 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>IN_PROGRESS · hợp lệ</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>DONE + hạ xuống IN_PROGRESS</t>
+          <t>Đánh dấu DONE, node mở khoá</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>IN_PROGRESS, xoá completedAt</t>
+          <t>DONE, ghi completedAt + nhật ký</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>st04</t>
+          <t>st02</t>
         </is>
       </c>
     </row>
@@ -4303,17 +4303,17 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>IN_PROGRESS · hợp lệ</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED + đánh dấu DONE (nhảy cóc)</t>
+          <t>Bỏ đánh dấu về NOT_STARTED</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>DONE, ghi completedAt + nhật ký</t>
+          <t>NOT_STARTED, không hỏi khoá</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>st05 · CẠNH MỚI PHỦ</t>
+          <t>st06 · CẠNH BỔ SUNG</t>
         </is>
       </c>
     </row>
@@ -4345,17 +4345,17 @@
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Chuyển hợp lệ</t>
+          <t>IN_PROGRESS · KHÔNG hợp lệ</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>IN_PROGRESS + bỏ đánh dấu</t>
+          <t>Đánh dấu DONE khi node BỊ KHOÁ</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
+          <t>Bị chặn 403, không lưu/ghi log</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -4370,7 +4370,7 @@
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>st06 · CẠNH MỚI PHỦ</t>
+          <t>st08</t>
         </is>
       </c>
     </row>
@@ -4387,17 +4387,17 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Chuyển KHÔNG hợp lệ</t>
+          <t>DONE · hợp lệ</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED + DONE khi node KHOÁ</t>
+          <t>Bỏ đánh dấu về NOT_STARTED</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Bị chặn 403, không lưu</t>
+          <t>NOT_STARTED, XOÁ completedAt</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -4412,7 +4412,7 @@
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>st07</t>
+          <t>st03</t>
         </is>
       </c>
     </row>
@@ -4429,17 +4429,17 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Chuyển KHÔNG hợp lệ</t>
+          <t>DONE · hợp lệ</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>IN_PROGRESS + DONE khi node KHOÁ</t>
+          <t>Hạ xuống IN_PROGRESS</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>Bị chặn 403, không lưu/ghi log</t>
+          <t>IN_PROGRESS, XOÁ completedAt</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -4454,7 +4454,7 @@
       </c>
       <c r="H14" s="8" t="inlineStr">
         <is>
-          <t>st08</t>
+          <t>st04</t>
         </is>
       </c>
     </row>
@@ -4541,12 +4541,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>NOT_STARTED</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Đánh dấu DONE (node mở)</t>
+          <t>Đánh dấu DONE (node mở, nhảy cóc)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -4575,27 +4575,27 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>NOT_STARTED</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Bỏ đánh dấu</t>
+          <t>Đánh dấu DONE khi node KHOÁ</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Có</t>
+          <t>Bị chặn (403)</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>KHÔNG</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>XOÁ completedAt</t>
+          <t>Không lưu gì</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
@@ -4609,19 +4609,19 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Đánh dấu DONE (node mở)</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>Hạ xuống IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
           <t>Có</t>
@@ -4629,7 +4629,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>XOÁ completedAt</t>
+          <t>Ghi completedAt + nhật ký</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr"/>
@@ -4643,19 +4643,19 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Bỏ đánh dấu</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
           <t>NOT_STARTED</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Đánh dấu DONE (node mở)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Có</t>
@@ -4663,7 +4663,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Ghi completedAt + nhật ký</t>
+          <t>Không hỏi khoá</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr"/>
@@ -4682,22 +4682,22 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Bỏ đánh dấu</t>
+          <t>Đánh dấu DONE khi node KHOÁ</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Có</t>
+          <t>Bị chặn (403)</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="inlineStr">
+        <is>
+          <t>KHÔNG</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Không hỏi khoá</t>
+          <t>Không lưu, không ghi log</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr"/>
@@ -4711,27 +4711,27 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Bỏ đánh dấu</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
           <t>NOT_STARTED</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Đánh dấu DONE khi node KHOÁ</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>Bị chặn (403)</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="inlineStr">
-        <is>
-          <t>KHÔNG</t>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>Không lưu gì</t>
+          <t>XOÁ completedAt</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr"/>
@@ -4745,27 +4745,27 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>Hạ xuống IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
           <t>IN_PROGRESS</t>
         </is>
       </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Đánh dấu DONE khi node KHOÁ</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Bị chặn (403)</t>
-        </is>
-      </c>
-      <c r="E25" s="11" t="inlineStr">
-        <is>
-          <t>KHÔNG</t>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Không lưu, không ghi log</t>
+          <t>XOÁ completedAt</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr"/>
@@ -4777,9 +4777,9 @@
           <t>9</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>___  ⟵ BẠN ĐIỀN</t>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -4815,7 +4815,7 @@
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>GỢI Ý dòng 9: còn MỘT trạng thái đầu nữa chưa được thử với node bị khoá. Nhìn cột Start State của dòng 7 và 8 — thiếu trạng thái nào trong ba trạng thái?</t>
+          <t>GỢI Ý dòng 9: bảng nhóm theo Start State, mỗi nhóm gồm 2 chuyển đổi hợp lệ + 1 chuyển đổi bị chặn. Nhóm NOT_STARTED và IN_PROGRESS đã đủ 3 dòng, nhóm DONE mới có 2. Vậy từ DONE, đánh dấu sang trạng thái nào thì bị chặn khi node khoá? Nhớ luật: chỉ chuyển VỀ NOT_STARTED là không bị kiểm khoá.</t>
         </is>
       </c>
     </row>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>8 case, phủ đủ 6 cạnh + 2 chặn</t>
+          <t>8 case, nhóm theo Start State</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
test(blackbox): hoàn thiện bảng chuyển trạng thái - 3 nhóm x 3 dòng
Thêm ST-09: từ DONE hạ về IN_PROGRESS khi node bị khoá -> chặn 403. Đây là
dòng cuối để bảng cân xứng: mỗi trạng thái xuất phát có đúng 2 chuyển đổi
hợp lệ và 1 chuyển đổi bị chặn.
  NOT_STARTED  dòng 1-3
  IN_PROGRESS  dòng 4-6
  DONE         dòng 7-9

Sáu dòng hợp lệ phủ trọn 6 cạnh của sơ đồ (3 trạng thái x 2 đích). Ba dòng
bị chặn kiểm chứng chốt chặn hoạt động nhất quán từ cả ba trạng thái.

Bỏ ô chừa ảnh sơ đồ, thay bằng ghi chú trỏ tới SoDo-ChuyenTrangThai.drawio.

Ghi chú thêm về tầng kiểm thử: giao diện roadmap chỉ có 4 nút nên 2 trong 6
cạnh không bấm được từ màn hình, nhưng cả 6 đều gọi được qua
POST /roadmap/progress. Ẩn nút là rào chắn mềm phía client, không phải bảo vệ
thật - nên vẫn phải kiểm thử đủ ở tầng dịch vụ.

Phần A: 32 test, không còn ô trống nào trong cả 4 sheet báo cáo.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -62,7 +62,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -94,11 +94,6 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -126,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -156,9 +151,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4049,7 +4041,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>COUNTA($A$7:$A$14)</f>
+        <f>COUNTA($A$7:$A$15)</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -4058,7 +4050,7 @@
         </is>
       </c>
       <c r="D4" s="4">
-        <f>COUNTIF($G$7:$G$14,"PASS")</f>
+        <f>COUNTIF($G$7:$G$15,"PASS")</f>
         <v/>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -4067,7 +4059,7 @@
         </is>
       </c>
       <c r="F4" s="4">
-        <f>COUNTIF($G$7:$G$14,"Chưa chạy")</f>
+        <f>COUNTIF($G$7:$G$15,"Chưa chạy")</f>
         <v/>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -4076,7 +4068,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>COUNTIF($G$7:$G$14,"KNOWN BUG")</f>
+        <f>COUNTIF($G$7:$G$15,"KNOWN BUG")</f>
         <v/>
       </c>
     </row>
@@ -4458,85 +4450,93 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>ST-A09</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>ProgressStateTransitionTest</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>DONE · KHÔNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Hạ về IN_PROGRESS khi node BỊ KHOÁ</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Bị chặn 403, không lưu</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>st09</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
         <is>
           <t>BẢNG CHUYỂN TRẠNG THÁI — mẫu slide 39</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Test Case No.</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Start State</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Event / Input</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>End State / Exp Output</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Hợp lệ</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>Tác dụng phụ kiểm chứng</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr"/>
-      <c r="H17" s="5" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>NOT_STARTED</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Đánh dấu IN_PROGRESS (node mở)</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Có</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>completedAt vẫn null</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr"/>
-      <c r="H18" s="6" t="inlineStr"/>
+      <c r="G18" s="5" t="inlineStr"/>
+      <c r="H18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -4546,12 +4546,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Đánh dấu DONE (node mở, nhảy cóc)</t>
+          <t>Đánh dấu IN_PROGRESS (node mở)</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Ghi completedAt + nhật ký</t>
+          <t>completedAt vẫn null</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr"/>
@@ -4570,7 +4570,7 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -4580,22 +4580,22 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Đánh dấu DONE khi node KHOÁ</t>
+          <t>Đánh dấu DONE (node mở, nhảy cóc)</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Bị chặn (403)</t>
-        </is>
-      </c>
-      <c r="E20" s="11" t="inlineStr">
-        <is>
-          <t>KHÔNG</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>Không lưu gì</t>
+          <t>Ghi completedAt + nhật ký</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr"/>
@@ -4604,32 +4604,32 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>NOT_STARTED</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Đánh dấu DONE (node mở)</t>
+          <t>Đánh dấu DONE khi node KHOÁ</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Có</t>
+          <t>Bị chặn (403)</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="inlineStr">
+        <is>
+          <t>KHÔNG</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>Ghi completedAt + nhật ký</t>
+          <t>Không lưu gì</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr"/>
@@ -4638,7 +4638,7 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -4648,12 +4648,12 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Bỏ đánh dấu</t>
+          <t>Đánh dấu DONE (node mở)</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -4663,7 +4663,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Không hỏi khoá</t>
+          <t>Ghi completedAt + nhật ký</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr"/>
@@ -4672,7 +4672,7 @@
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -4682,22 +4682,22 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Đánh dấu DONE khi node KHOÁ</t>
+          <t>Bỏ đánh dấu</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Bị chặn (403)</t>
-        </is>
-      </c>
-      <c r="E23" s="11" t="inlineStr">
-        <is>
-          <t>KHÔNG</t>
+          <t>NOT_STARTED</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>Không lưu, không ghi log</t>
+          <t>Không hỏi khoá</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr"/>
@@ -4706,32 +4706,32 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Bỏ đánh dấu</t>
+          <t>Đánh dấu DONE khi node KHOÁ</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>NOT_STARTED</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Có</t>
+          <t>Bị chặn (403)</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="inlineStr">
+        <is>
+          <t>KHÔNG</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>XOÁ completedAt</t>
+          <t>Không lưu, không ghi log</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr"/>
@@ -4740,7 +4740,7 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
@@ -4750,12 +4750,12 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Hạ xuống IN_PROGRESS</t>
+          <t>Bỏ đánh dấu</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>NOT_STARTED</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -4774,7 +4774,7 @@
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
@@ -4782,68 +4782,98 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
-        <is>
-          <t>___  ⟵ BẠN ĐIỀN</t>
-        </is>
-      </c>
-      <c r="D26" s="12" t="inlineStr">
-        <is>
-          <t>___  ⟵ BẠN ĐIỀN</t>
-        </is>
-      </c>
-      <c r="E26" s="11" t="inlineStr">
-        <is>
-          <t>KHÔNG</t>
-        </is>
-      </c>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>___  ⟵ BẠN ĐIỀN</t>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>Hạ xuống IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>XOÁ completedAt</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr"/>
       <c r="H26" s="6" t="inlineStr"/>
     </row>
-    <row r="28" ht="34" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>TIÊU CHÍ ĐỦ của kỹ thuật này: phủ hết CẠNH của sơ đồ. Ba trạng thái sinh ra 3 × 2 = 6 cặp có thứ tự, tức 6 cạnh. Dòng 1–6 phủ đủ 6 cạnh đó. Dòng 7–8 là chuyển đổi bị chặn.</t>
-        </is>
-      </c>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Hạ về IN_PROGRESS khi node KHOÁ</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Bị chặn (403)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="inlineStr">
+        <is>
+          <t>KHÔNG</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>Không lưu gì</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr"/>
+      <c r="H27" s="6" t="inlineStr"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>GỢI Ý dòng 9: bảng nhóm theo Start State, mỗi nhóm gồm 2 chuyển đổi hợp lệ + 1 chuyển đổi bị chặn. Nhóm NOT_STARTED và IN_PROGRESS đã đủ 3 dòng, nhóm DONE mới có 2. Vậy từ DONE, đánh dấu sang trạng thái nào thì bị chặn khi node khoá? Nhớ luật: chỉ chuyển VỀ NOT_STARTED là không bị kiểm khoá.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>SƠ ĐỒ TRẠNG THÁI</t>
-        </is>
-      </c>
-      <c r="B30" s="12" t="inlineStr">
-        <is>
-          <t>[ CHÈN ẢNH SƠ ĐỒ BẠN VẼ VÀO ĐÂY ]  ⟵ BẠN ĐIỀN</t>
+          <t>TIÊU CHÍ ĐỦ của kỹ thuật này: phủ hết CẠNH của sơ đồ. Ba trạng thái sinh ra 3 × 2 = 6 cặp có thứ tự, tức 6 cạnh. Dòng 1–6 phủ đủ 6 cạnh đó. Dòng 7–8 là chuyển đổi bị chặn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>CẤU TRÚC BẢNG: nhóm theo Start State, mỗi nhóm đúng 3 dòng gồm 2 chuyển đổi hợp lệ và 1 chuyển đổi bị chặn khi node khoá. Sáu dòng hợp lệ phủ trọn 6 cạnh của sơ đồ (3 trạng thái x 2 đích = 6). Ba dòng bị chặn kiểm chứng chốt chặn hoạt động từ cả ba trạng thái xuất phát.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="34" customHeight="1">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>LƯU Ý VỀ TẦNG KIỂM THỬ: bảng này thiết kế ở TẦNG DỊCH VỤ, nơi luật nghiệp vụ thực sự được thi hành. Giao diện roadmap chỉ có 4 nút (NOT_STARTED→IN_PROGRESS, IN_PROGRESS→DONE, IN_PROGRESS→NOT_STARTED, DONE→IN_PROGRESS), tức 2 trong 6 cạnh không bấm được từ màn hình. Nhưng cả 6 đều gọi được qua POST /roadmap/progress, nên vẫn phải kiểm thử đủ — ẩn nút chỉ là rào chắn mềm phía client, không phải bảo vệ thật.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="34" customHeight="1">
       <c r="A32" s="10" t="inlineStr">
         <is>
-          <t>Sơ đồ cần: 3 ô trạng thái, 6 mũi tên chuyển, và ghi chú mũi tên nào bị chặn khi node khoá. Vẽ tay chụp ảnh cũng được.</t>
+          <t>SƠ ĐỒ TRẠNG THÁI: xem tệp SoDo-ChuyenTrangThai.drawio ở thư mục gốc dự án — 3 trạng thái, đủ 6 cạnh chuyển, phân biệt bằng màu: đỏ nét đứt là chuyển đổi bị chặn khi node khoá, xanh nét liền là luôn được phép.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A28:H28"/>
+  <mergeCells count="5">
+    <mergeCell ref="A30:H30"/>
+    <mergeCell ref="A29:H29"/>
     <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4974,12 +5004,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>$A$7:$A$14</t>
+          <t>$A$7:$A$15</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>8 case, nhóm theo Start State</t>
+          <t>9 case, nhóm theo Start State (3 nhóm x 3 dòng)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(report): bổ sung 6 case BVA dung lượng tệp còn thiếu trong báo cáo
Sheet 01 chỉ liệt kê 27 case của RegisterFormDTOBvaTest, bỏ sót toàn bộ 6 case
của OnboardingFileSizeBvaTest dù test đã tồn tại và pass từ trước.

Bổ sung:
- 6 case dung lượng tệp bảng điểm (0 byte, 1 byte, 5MB, 10MB-1, 10MB, 10MB+1)
- Dòng V5 trong bảng thiết kế, nhãn biên B19-B24
- Sửa mô tả sheet: BVA áp cho 2 chức năng chứ không riêng đăng ký

Sau bổ sung: 46 case (33 BVA + 13 EP), nhãn V1-V5, X1-X11, B1-B24 đều liên tục.
Thứ tự dòng trong bảng thiết kế khớp thứ tự nhãn V1..V5.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H60"/>
+  <dimension ref="A1:H67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -540,7 +540,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Phân hoạch lớp tương đương và phân tích giá trị biên trên form đăng ký (RegisterFormDTO). Bảng thiết kế theo mẫu slide 32.</t>
+          <t>Phân hoạch lớp tương đương và phân tích giá trị biên trên 2 chức năng: đăng ký tài khoản (RegisterFormDTO) và tải lên bảng điểm. Bảng thiết kế theo mẫu slide 32.</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>COUNTA($A$7:$A$46)</f>
+        <f>COUNTA($A$7:$A$52)</f>
         <v/>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="D4" s="4">
-        <f>COUNTIF($G$7:$G$46,"PASS")</f>
+        <f>COUNTIF($G$7:$G$52,"PASS")</f>
         <v/>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="F4" s="4">
-        <f>COUNTIF($G$7:$G$46,"Chưa chạy")</f>
+        <f>COUNTIF($G$7:$G$52,"Chưa chạy")</f>
         <v/>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="H4" s="4">
-        <f>COUNTIF($G$7:$G$46,"KNOWN BUG")</f>
+        <f>COUNTIF($G$7:$G$52,"KNOWN BUG")</f>
         <v/>
       </c>
     </row>
@@ -1761,22 +1761,22 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>EP-01</t>
+          <t>BVA-28</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>password · lớp hợp lệ</t>
+          <t>Tệp bảng điểm · Standard BVA</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
         <is>
-          <t>V1 — "matkhau123" (10 ký tự)</t>
+          <t>min = 0 byte</t>
         </is>
       </c>
       <c r="E34" s="8" t="inlineStr">
@@ -1796,34 +1796,34 @@
       </c>
       <c r="H34" s="8" t="inlineStr">
         <is>
-          <t>v1_lopHopLe_duocChapNhan</t>
+          <t>B19</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>EP-02</t>
+          <t>BVA-29</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>password · lớp không hợp lệ</t>
+          <t>Tệp bảng điểm · Standard BVA</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>X1 — "abc" (dưới 6 ký tự)</t>
+          <t>min+1 = 1 byte</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Size)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -1838,34 +1838,34 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>x1_duoiSauKyTu_biTuChoi</t>
+          <t>B20</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>EP-03</t>
+          <t>BVA-30</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>password · lớp không hợp lệ</t>
+          <t>Tệp bảng điểm · Standard BVA</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
         <is>
-          <t>X2 — 31 ký tự</t>
+          <t>nominal = 5 MB</t>
         </is>
       </c>
       <c r="E36" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Size)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F36" s="8" t="inlineStr">
@@ -1880,34 +1880,34 @@
       </c>
       <c r="H36" s="8" t="inlineStr">
         <is>
-          <t>x2_tren30KyTu_biTuChoi</t>
+          <t>B21</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>EP-04</t>
+          <t>BVA-31</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>password · lớp không hợp lệ</t>
+          <t>Tệp bảng điểm · Standard BVA</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>X3 — 8 dấu cách</t>
+          <t>max-1 = 10MB − 1 byte</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@NotBlank)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -1922,34 +1922,34 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>LỚP BVA KHÔNG CHẠM TỚI</t>
+          <t>B22</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>EP-05</t>
+          <t>BVA-32</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C38" s="8" t="inlineStr">
         <is>
-          <t>password · lớp không hợp lệ</t>
+          <t>Tệp bảng điểm · Standard BVA</t>
         </is>
       </c>
       <c r="D38" s="8" t="inlineStr">
         <is>
-          <t>X4 — null</t>
+          <t>max = 10 MB</t>
         </is>
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@NotBlank)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F38" s="8" t="inlineStr">
@@ -1964,34 +1964,34 @@
       </c>
       <c r="H38" s="8" t="inlineStr">
         <is>
-          <t>x4_null_biTuChoi</t>
+          <t>B23</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>EP-06</t>
+          <t>BVA-33</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>fullName · lớp hợp lệ</t>
+          <t>Tệp bảng điểm · Robustness BVA</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>V2 — "Nguyen Van A"</t>
+          <t>max+1 = 10MB + 1 byte</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Được chấp nhận</t>
+          <t>Bị từ chối (vượt max-file-size)</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2006,14 +2006,14 @@
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>v2_fullName_lopHopLe</t>
+          <t>B24</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>EP-07</t>
+          <t>EP-01</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
@@ -2023,17 +2023,17 @@
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>fullName · lớp không hợp lệ</t>
+          <t>password · lớp hợp lệ</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
         <is>
-          <t>X5 — 101 ký tự</t>
+          <t>V1 — "matkhau123" (10 ký tự)</t>
         </is>
       </c>
       <c r="E40" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Size)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F40" s="8" t="inlineStr">
@@ -2048,14 +2048,14 @@
       </c>
       <c r="H40" s="8" t="inlineStr">
         <is>
-          <t>x5_fullName_tren100KyTu</t>
+          <t>v1_lopHopLe_duocChapNhan</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>EP-08</t>
+          <t>EP-02</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>fullName · lớp không hợp lệ</t>
+          <t>password · lớp không hợp lệ</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>X6 — toàn khoảng trắng</t>
+          <t>X1 — "abc" (dưới 6 ký tự)</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@NotBlank)</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -2090,14 +2090,14 @@
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>x6_fullName_toanKhoangTrang</t>
+          <t>x1_duoiSauKyTu_biTuChoi</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>EP-09</t>
+          <t>EP-03</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
@@ -2107,17 +2107,17 @@
       </c>
       <c r="C42" s="8" t="inlineStr">
         <is>
-          <t>fullName · lớp không hợp lệ</t>
+          <t>password · lớp không hợp lệ</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
         <is>
-          <t>X7 — null</t>
+          <t>X2 — 31 ký tự</t>
         </is>
       </c>
       <c r="E42" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@NotBlank)</t>
+          <t>Bị từ chối (@Size)</t>
         </is>
       </c>
       <c r="F42" s="8" t="inlineStr">
@@ -2132,14 +2132,14 @@
       </c>
       <c r="H42" s="8" t="inlineStr">
         <is>
-          <t>x7_fullName_null</t>
+          <t>x2_tren30KyTu_biTuChoi</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>EP-10</t>
+          <t>EP-04</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
@@ -2149,17 +2149,17 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>email · lớp hợp lệ</t>
+          <t>password · lớp không hợp lệ</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>V3 + V4 — "sinhvien@uth.edu.vn"</t>
+          <t>X3 — 8 dấu cách</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Được chấp nhận</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
@@ -2174,14 +2174,14 @@
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Một test phủ CẢ HAI lớp hợp lệ: độ dài (V3) và định dạng (V4)</t>
+          <t>LỚP BVA KHÔNG CHẠM TỚI</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>EP-11</t>
+          <t>EP-05</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
@@ -2191,17 +2191,17 @@
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>email · lớp không hợp lệ</t>
+          <t>password · lớp không hợp lệ</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>X8 — "khong-phai-email"</t>
+          <t>X4 — null</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Email)</t>
+          <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -2216,14 +2216,14 @@
       </c>
       <c r="H44" s="8" t="inlineStr">
         <is>
-          <t>x8_email_saiDinhDang</t>
+          <t>x4_null_biTuChoi</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>EP-12</t>
+          <t>EP-06</t>
         </is>
       </c>
       <c r="B45" s="6" t="inlineStr">
@@ -2233,17 +2233,17 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>email · lớp không hợp lệ</t>
+          <t>fullName · lớp hợp lệ</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>X9 — 153 ký tự</t>
+          <t>V2 — "Nguyen Van A"</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Bị từ chối (@Size)</t>
+          <t>Được chấp nhận</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -2258,119 +2258,371 @@
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>x9_email_tren150KyTu</t>
+          <t>v2_fullName_lopHopLe</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
+          <t>EP-07</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="inlineStr">
+        <is>
+          <t>fullName · lớp không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t>X5 — 101 ký tự</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối (@Size)</t>
+        </is>
+      </c>
+      <c r="F46" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G46" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H46" s="8" t="inlineStr">
+        <is>
+          <t>x5_fullName_tren100KyTu</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>EP-08</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>fullName · lớp không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>X6 — toàn khoảng trắng</t>
+        </is>
+      </c>
+      <c r="E47" s="6" t="inlineStr">
+        <is>
+          <t>Bị từ chối (@NotBlank)</t>
+        </is>
+      </c>
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>x6_fullName_toanKhoangTrang</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>EP-09</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>fullName · lớp không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>X7 — null</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối (@NotBlank)</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H48" s="8" t="inlineStr">
+        <is>
+          <t>x7_fullName_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>EP-10</t>
+        </is>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>email · lớp hợp lệ</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr">
+        <is>
+          <t>V3 + V4 — "sinhvien@uth.edu.vn"</t>
+        </is>
+      </c>
+      <c r="E49" s="6" t="inlineStr">
+        <is>
+          <t>Được chấp nhận</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>Một test phủ CẢ HAI lớp hợp lệ: độ dài (V3) và định dạng (V4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>EP-11</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>email · lớp không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>X8 — "khong-phai-email"</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>Bị từ chối (@Email)</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H50" s="8" t="inlineStr">
+        <is>
+          <t>x8_email_saiDinhDang</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>EP-12</t>
+        </is>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>email · lớp không hợp lệ</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>X9 — 153 ký tự</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="inlineStr">
+        <is>
+          <t>Bị từ chối (@Size)</t>
+        </is>
+      </c>
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>x9_email_tren150KyTu</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
           <t>EP-13</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t>RegisterEquivalencePartitionTest</t>
         </is>
       </c>
-      <c r="C46" s="8" t="inlineStr">
+      <c r="C52" s="8" t="inlineStr">
         <is>
           <t>email · lớp không hợp lệ</t>
         </is>
       </c>
-      <c r="D46" s="8" t="inlineStr">
+      <c r="D52" s="8" t="inlineStr">
         <is>
           <t>X10 — null</t>
         </is>
       </c>
-      <c r="E46" s="8" t="inlineStr">
+      <c r="E52" s="8" t="inlineStr">
         <is>
           <t>Bị từ chối (@NotBlank)</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
-        <is>
-          <t>Đã chạy, đúng như mong đợi</t>
-        </is>
-      </c>
-      <c r="G46" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-      <c r="H46" s="8" t="inlineStr">
+      <c r="F52" s="8" t="inlineStr">
+        <is>
+          <t>Đã chạy, đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="H52" s="8" t="inlineStr">
         <is>
           <t>x10_email_null</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="24" customHeight="1">
-      <c r="A48" s="9" t="inlineStr">
+    <row r="54" ht="24" customHeight="1">
+      <c r="A54" s="9" t="inlineStr">
         <is>
           <t>BẢNG THIẾT KẾ — mẫu slide 32 (Conditions / Valid / Invalid / Boundaries)</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Conditions</t>
         </is>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>Valid Partitions</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Invalid Partitions</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F55" s="5" t="inlineStr">
         <is>
           <t>Valid Boundaries (Standard)</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="H49" s="5" t="inlineStr">
+      <c r="H55" s="5" t="inlineStr">
         <is>
           <t>Robustness (min-1 / max+1)</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="62" customHeight="1">
-      <c r="A50" s="6" t="inlineStr">
+    <row r="56" ht="62" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B50" s="6" t="inlineStr">
+      <c r="B56" s="6" t="inlineStr">
         <is>
           <t>6–30 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C50" s="6" t="inlineStr">
+      <c r="C56" s="6" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="D50" s="6" t="inlineStr">
+      <c r="D56" s="6" t="inlineStr">
         <is>
           <t>&lt; 6 ký tự
 &gt; 30 ký tự
@@ -2378,7 +2630,7 @@
 null</t>
         </is>
       </c>
-      <c r="E50" s="6" t="inlineStr">
+      <c r="E56" s="6" t="inlineStr">
         <is>
           <t>X1
 X2
@@ -2386,197 +2638,241 @@
 X4</t>
         </is>
       </c>
-      <c r="F50" s="6" t="inlineStr">
+      <c r="F56" s="6" t="inlineStr">
         <is>
           <t>6, 7, 18, 29, 30</t>
         </is>
       </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>B1–B5</t>
         </is>
       </c>
-      <c r="H50" s="6" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>5 và 31
 (B6, B7)</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="62" customHeight="1">
-      <c r="A51" s="6" t="inlineStr">
+    <row r="57" ht="62" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="B51" s="6" t="inlineStr">
+      <c r="B57" s="6" t="inlineStr">
         <is>
           <t>1–100 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>&gt; 100 ký tự
 toàn khoảng trắng
 null</t>
         </is>
       </c>
-      <c r="E51" s="6" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>X5
 X6
 X7</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>1, 2, 50, 99, 100</t>
         </is>
       </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="G57" s="6" t="inlineStr">
         <is>
           <t>B8–B12</t>
         </is>
       </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>rỗng (= min−1) và 101
 (B13, B14)</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="62" customHeight="1">
-      <c r="A52" s="6" t="inlineStr">
+    <row r="58" ht="62" customHeight="1">
+      <c r="A58" s="6" t="inlineStr">
         <is>
           <t>email — điều kiện ĐỘ DÀI</t>
         </is>
       </c>
-      <c r="B52" s="6" t="inlineStr">
+      <c r="B58" s="6" t="inlineStr">
         <is>
           <t>≤ 150 ký tự</t>
         </is>
       </c>
-      <c r="C52" s="6" t="inlineStr">
+      <c r="C58" s="6" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D58" s="6" t="inlineStr">
         <is>
           <t>&gt; 150 ký tự</t>
         </is>
       </c>
-      <c r="E52" s="6" t="inlineStr">
+      <c r="E58" s="6" t="inlineStr">
         <is>
           <t>X9</t>
         </is>
       </c>
-      <c r="F52" s="6" t="inlineStr">
+      <c r="F58" s="6" t="inlineStr">
         <is>
           <t>75, 149, 150
 (KHÔNG có biên dưới)</t>
         </is>
       </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="G58" s="6" t="inlineStr">
         <is>
           <t>B15–B17</t>
         </is>
       </c>
-      <c r="H52" s="6" t="inlineStr">
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>151
 (B18, chỉ có max+1)</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="62" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="59" ht="62" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
         <is>
           <t>email — điều kiện ĐỊNH DẠNG</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B59" s="6" t="inlineStr">
         <is>
           <t>đúng định dạng email</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>sai định dạng
 null / rỗng</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>X8
 X10</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
         <is>
           <t>(không áp dụng —
 miền rời rạc)</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G59" s="6" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>(không áp dụng)</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="34" customHeight="1">
-      <c r="A55" s="10" t="inlineStr">
+    <row r="60" ht="62" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm — DUNG LƯỢNG</t>
+        </is>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>0 đến 10 MB</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>V5</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 10 MB</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="inlineStr">
+        <is>
+          <t>X11</t>
+        </is>
+      </c>
+      <c r="F60" s="6" t="inlineStr">
+        <is>
+          <t>0, 1 byte, 5 MB,
+10MB−1, 10 MB</t>
+        </is>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>B19–B23</t>
+        </is>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
+        <is>
+          <t>10MB + 1 byte
+(B24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="34" customHeight="1">
+      <c r="A62" s="10" t="inlineStr">
         <is>
           <t>GỢI Ý ô trống: khoảng hợp lệ của password là [6, 30]. Robustness BVA thêm đúng hai giá trị ngay NGOÀI biên — min−1 và max+1. Vậy hai số đó là gì? (xem lại dòng fullName và email ở trên để thấy quy luật).</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="34" customHeight="1">
-      <c r="A56" s="10" t="inlineStr">
+    <row r="63" ht="34" customHeight="1">
+      <c r="A63" s="10" t="inlineStr">
         <is>
           <t>LƯU Ý QUAN TRỌNG khi thuyết trình: cột 'Valid Boundaries (Standard)' chỉ chứa giá trị HỢP LỆ — công thức 4n+1. Đối chiếu slide 29: khoảng [2, 64] cho ra 2, 3, 63, 64, 33; slide 31: khoảng [500, 9000] cho ra 500, 501, 4750, 8999, 9000. Không giá trị nào vượt ra ngoài khoảng. Giá trị ngoài biên thuộc cột Robustness (6n+1).</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="34" customHeight="1">
-      <c r="A57" s="10" t="inlineStr">
+    <row r="64" ht="34" customHeight="1">
+      <c r="A64" s="10" t="inlineStr">
         <is>
           <t>QUY TẮC GỘP LỚP HỢP LỆ: một test case có thể phủ NHIỀU lớp hợp lệ cùng lúc — EP-10 dùng "sinhvien@uth.edu.vn" vừa thoả V3 (độ dài ≤ 150) vừa thoả V4 (đúng định dạng), nên phủ luôn cả hai. Ngược lại, lớp KHÔNG hợp lệ phải tách riêng từng test: nếu một test vừa sai định dạng vừa quá 150 ký tự thì ràng buộc nào bắt trước sẽ CHE MẤT ràng buộc kia, không biết cái còn lại có được kiểm hay không. Đây cũng là lý do bạn Quân dùng validateProperty(dto, "password") thay vì validate(dto) — để cô lập đúng một trường.</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="34" customHeight="1">
-      <c r="A58" s="10" t="inlineStr">
+    <row r="65" ht="34" customHeight="1">
+      <c r="A65" s="10" t="inlineStr">
         <is>
           <t>VÌ SAO EMAIL KHÔNG CÓ BIÊN DƯỚI: ràng buộc của email là @NotBlank + @Email + @Size(max = 150) — CHỈ khai max, không khai min. Đã kiểm chứng thực nghiệm: a@b (3 ký tự) và a@b.c (5 ký tự) đều được chấp nhận. Vì thế Robustness của email chỉ có max+1 = 151, không có min−1. Khác với password (@Size khai min=6 nên min−1 = 5 là giá trị không hợp lệ thật) và fullName (biên dưới do @NotBlank sinh ra nên chuỗi rỗng chính là min−1).</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="34" customHeight="1">
-      <c r="A59" s="10" t="inlineStr">
+    <row r="66" ht="34" customHeight="1">
+      <c r="A66" s="10" t="inlineStr">
         <is>
           <t>VÌ SAO TÁCH EMAIL LÀM HAI DÒNG: theo mẫu slide 29, một trường có thể mang nhiều điều kiện độc lập — Customer name được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên; điều kiện ĐỊNH DẠNG là miền rời rạc (đúng/sai) nên chỉ phân lớp được, không có biên.</t>
         </is>
       </c>
     </row>
-    <row r="60" ht="34" customHeight="1">
-      <c r="A60" s="10" t="inlineStr">
+    <row r="67" ht="34" customHeight="1">
+      <c r="A67" s="10" t="inlineStr">
         <is>
           <t>PHÁT HIỆN — lớp X3: chuỗi 8 dấu cách có độ dài 8 nên THOẢ MÃN @Size(min=6, max=30), nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên kỹ thuật giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện ra. Đây là bằng chứng hai kỹ thuật bổ sung cho nhau chứ không thay thế nhau.</t>
         </is>
@@ -2584,13 +2880,13 @@
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A56:H56"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A55:H55"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="A57:H57"/>
-    <mergeCell ref="A60:H60"/>
-    <mergeCell ref="A58:H58"/>
+    <mergeCell ref="A67:H67"/>
+    <mergeCell ref="A62:H62"/>
+    <mergeCell ref="A65:H65"/>
+    <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A64:H64"/>
+    <mergeCell ref="A66:H66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4938,12 +5234,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>$A$7:$A$47</t>
+          <t>$A$7:$A$52</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>41 case: 28 BVA + 13 EP</t>
+          <t>46 case: 33 BVA (27 đăng ký + 6 tệp) + 13 EP</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(report): gắn nhãn phân biệt nhật ký chạy test với bảng thiết kế
Mỗi sheet có hai loại bảng khác hẳn nhau về mục đích nhưng trước đây không có
gì phân biệt: danh sách case ở trên là bằng chứng ĐÃ CHẠY (mẫu chung của nhóm,
không có trong slide), các bảng bên dưới là THIẾT KẾ test theo slide 23/32/44/39.

Thêm thanh nhãn ở dòng 5 của cả 4 sheet dữ liệu để người đọc báo cáo tự phân
biệt được, không cần người trình bày giải thích.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,6 +168,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -599,6 +602,13 @@
         <v/>
       </c>
     </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NHẬT KÝ CHẠY TEST — danh sách case đã thực thi (bằng chứng thi hành, mẫu chung của nhóm). Bảng THIẾT KẾ theo slide nằm bên dưới danh sách này.</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -4592,8 +4602,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A109:H109"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A99:H99"/>
@@ -4679,6 +4690,13 @@
         <v/>
       </c>
     </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NHẬT KÝ CHẠY TEST — danh sách case đã thực thi (bằng chứng thi hành, mẫu chung của nhóm). Bảng THIẾT KẾ theo slide nằm bên dưới danh sách này.</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -5354,11 +5372,12 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A31:H31"/>
-    <mergeCell ref="A21:H21"/>
     <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A14:H14"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5435,6 +5454,13 @@
         <v/>
       </c>
     </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NHẬT KÝ CHẠY TEST — danh sách case đã thực thi (bằng chứng thi hành, mẫu chung của nhóm). Bảng THIẾT KẾ theo slide nằm bên dưới danh sách này.</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -6001,12 +6027,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A29:H29"/>
     <mergeCell ref="A20:H20"/>
     <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A31:H31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6084,6 +6111,13 @@
         <v/>
       </c>
     </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="15" t="inlineStr">
+        <is>
+          <t>NHẬT KÝ CHẠY TEST — danh sách case đã thực thi (bằng chứng thi hành, mẫu chung của nhóm). Bảng THIẾT KẾ theo slide nằm bên dưới danh sách này.</t>
+        </is>
+      </c>
+    </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -6880,9 +6914,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A30:H30"/>
     <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A5:H5"/>
     <mergeCell ref="A32:H32"/>
     <mergeCell ref="A31:H31"/>
     <mergeCell ref="A17:H17"/>

</xml_diff>

<commit_message>
docs(report): giải thích vì sao cột Input có dòng ghi 1 trường, có dòng ghi 3
Các dòng BVA-xx/EP-xx dùng validateProperty nên chỉ một trường tham gia kết
quả - đây là cách phân tích biên theo TỪNG TRƯỜNG như slide 29-31 (ví dụ
Loan application).

Các dòng SBVA-xx dùng validate(dto) nên cả ba trường đều tham gia và phải ghi
đủ, hai trường không xét đặt ở nom - đúng cấu trúc bảng Standard BVA slide 23.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014bubSB5r22QGnSRDvVzw4d
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -537,7 +537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3381,256 +3381,231 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="24" customHeight="1">
-      <c r="A73" s="12" t="inlineStr">
+    <row r="72" ht="48" customHeight="1">
+      <c r="A72" s="10" t="inlineStr">
+        <is>
+          <t>CÁCH ĐỌC CỘT INPUT: các dòng BVA-xx và EP-xx chỉ ghi MỘT trường vì chúng dùng validateProperty(dto, "tên trường") — chỉ kiểm ràng buộc của trường đó, hai trường còn lại không tham gia kết quả nên không ghi. Đây là cách phân tích biên theo TỪNG TRƯỜNG như slide 29-31 của ví dụ Loan application. Các dòng SBVA-xx ghi ĐỦ BA trường vì dùng validate(dto) — kiểm cả form nên cả ba giá trị đều ảnh hưởng kết quả; trường đang xét đặt ở giá trị biên, hai trường kia đặt ở nom, đúng cấu trúc bảng Standard BVA slide 23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="24" customHeight="1"/>
+    <row r="74" ht="30" customHeight="1">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t>BẢNG 1 — ĐỊNH NGHĨA GIÁ TRỊ BIÊN CỦA TỪNG BIẾN (phần ghi chú bên trái slide 23)</t>
         </is>
       </c>
     </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="5" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>Giá trị</t>
         </is>
       </c>
-      <c r="B74" s="5" t="inlineStr">
+      <c r="B75" s="5" t="inlineStr">
         <is>
           <t>fullName (số ký tự)</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
+      <c r="C75" s="5" t="inlineStr">
         <is>
           <t>email (số ký tự)</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>password (số ký tự)</t>
         </is>
       </c>
-      <c r="E74" s="5" t="inlineStr"/>
-      <c r="F74" s="5" t="inlineStr"/>
-      <c r="G74" s="5" t="inlineStr"/>
-      <c r="H74" s="5" t="inlineStr">
+      <c r="E75" s="5" t="inlineStr"/>
+      <c r="F75" s="5" t="inlineStr"/>
+      <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="5" t="inlineStr">
         <is>
           <t>Ghi chú</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
-        <is>
-          <t>min</t>
-        </is>
-      </c>
-      <c r="B75" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C75" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="D75" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E75" s="6" t="inlineStr"/>
-      <c r="F75" s="6" t="inlineStr"/>
-      <c r="G75" s="6" t="inlineStr"/>
-      <c r="H75" s="6" t="inlineStr">
-        <is>
-          <t>giá trị nhỏ nhất hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>min+</t>
+          <t>min</t>
         </is>
       </c>
       <c r="B76" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C76" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D76" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E76" s="6" t="inlineStr"/>
       <c r="F76" s="6" t="inlineStr"/>
       <c r="G76" s="6" t="inlineStr"/>
       <c r="H76" s="6" t="inlineStr">
         <is>
-          <t>ngay trên min</t>
+          <t>giá trị nhỏ nhất hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>nom</t>
+          <t>min+</t>
         </is>
       </c>
       <c r="B77" s="4" t="n">
-        <v>50</v>
+        <v>2</v>
       </c>
       <c r="C77" s="4" t="n">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="D77" s="4" t="n">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="E77" s="6" t="inlineStr"/>
       <c r="F77" s="6" t="inlineStr"/>
       <c r="G77" s="6" t="inlineStr"/>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>giá trị điển hình, giữa miền</t>
+          <t>ngay trên min</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>max-</t>
+          <t>nom</t>
         </is>
       </c>
       <c r="B78" s="4" t="n">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="C78" s="4" t="n">
-        <v>149</v>
+        <v>75</v>
       </c>
       <c r="D78" s="4" t="n">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="E78" s="6" t="inlineStr"/>
       <c r="F78" s="6" t="inlineStr"/>
       <c r="G78" s="6" t="inlineStr"/>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>ngay dưới max</t>
+          <t>giá trị điển hình, giữa miền</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>max-</t>
         </is>
       </c>
       <c r="B79" s="4" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C79" s="4" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D79" s="4" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E79" s="6" t="inlineStr"/>
       <c r="F79" s="6" t="inlineStr"/>
       <c r="G79" s="6" t="inlineStr"/>
       <c r="H79" s="6" t="inlineStr">
         <is>
+          <t>ngay dưới max</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="C80" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="D80" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E80" s="6" t="inlineStr"/>
+      <c r="F80" s="6" t="inlineStr"/>
+      <c r="G80" s="6" t="inlineStr"/>
+      <c r="H80" s="6" t="inlineStr">
+        <is>
           <t>giá trị lớn nhất hợp lệ</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="34" customHeight="1">
-      <c r="A81" s="10" t="inlineStr">
+    <row r="81" ht="34" customHeight="1"/>
+    <row r="82" ht="24" customHeight="1">
+      <c r="A82" s="10" t="inlineStr">
         <is>
           <t>Ràng buộc gốc: fullName @NotBlank @Size(max=100) · email @NotBlank @Email @Size(max=150) · password @NotBlank @Size(min=6, max=30). Biên dưới của fullName do @NotBlank sinh ra (chuỗi rỗng bị chặn nên min = 1). Biên dưới của email là BIÊN VẬN HÀNH — độ dài email quy ước ngắn nhất a@b.co — vì @Size không khai min.</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="24" customHeight="1">
-      <c r="A82" s="12" t="inlineStr">
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="12" t="inlineStr">
         <is>
           <t>BẢNG 2 — STANDARD BVA TEST CASES (mẫu slide 23) · số case = 4n + 1 = 4×3 + 1 = 13</t>
         </is>
       </c>
     </row>
-    <row r="83" ht="30" customHeight="1">
-      <c r="A83" s="5" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B83" s="5" t="inlineStr">
+      <c r="B84" s="5" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
+      <c r="C84" s="5" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D83" s="5" t="inlineStr">
+      <c r="D84" s="5" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="E83" s="5" t="inlineStr">
+      <c r="E84" s="5" t="inlineStr">
         <is>
           <t>Biến đang xét</t>
         </is>
       </c>
-      <c r="F83" s="5" t="inlineStr">
+      <c r="F84" s="5" t="inlineStr">
         <is>
           <t>Expected Output</t>
         </is>
       </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="G84" s="5" t="inlineStr">
         <is>
           <t>Kết quả thực tế</t>
         </is>
       </c>
-      <c r="H83" s="5" t="inlineStr">
+      <c r="H84" s="5" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B84" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C84" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="D84" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="E84" s="6" t="inlineStr">
-        <is>
-          <t>password = min</t>
-        </is>
-      </c>
-      <c r="F84" s="6" t="inlineStr">
-        <is>
-          <t>Hợp lệ</t>
-        </is>
-      </c>
-      <c r="G84" s="6" t="inlineStr">
-        <is>
-          <t>Đúng như mong đợi</t>
-        </is>
-      </c>
-      <c r="H84" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B85" s="4" t="n">
         <v>50</v>
@@ -3639,11 +3614,11 @@
         <v>75</v>
       </c>
       <c r="D85" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>password = min+</t>
+          <t>password = min</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -3664,7 +3639,7 @@
     </row>
     <row r="86">
       <c r="A86" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B86" s="4" t="n">
         <v>50</v>
@@ -3672,12 +3647,12 @@
       <c r="C86" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D86" s="4" t="n">
-        <v>18</v>
+      <c r="D86" s="13" t="n">
+        <v>7</v>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>TẤT CẢ nominal</t>
+          <t>password = min+</t>
         </is>
       </c>
       <c r="F86" s="6" t="inlineStr">
@@ -3698,7 +3673,7 @@
     </row>
     <row r="87">
       <c r="A87" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B87" s="4" t="n">
         <v>50</v>
@@ -3706,12 +3681,12 @@
       <c r="C87" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D87" s="13" t="n">
-        <v>29</v>
+      <c r="D87" s="4" t="n">
+        <v>18</v>
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>password = max-</t>
+          <t>TẤT CẢ nominal</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
@@ -3732,7 +3707,7 @@
     </row>
     <row r="88">
       <c r="A88" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B88" s="4" t="n">
         <v>50</v>
@@ -3741,11 +3716,11 @@
         <v>75</v>
       </c>
       <c r="D88" s="13" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>password = max</t>
+          <t>password = max-</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
@@ -3766,20 +3741,20 @@
     </row>
     <row r="89">
       <c r="A89" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B89" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C89" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="D89" s="4" t="n">
-        <v>18</v>
+      <c r="C89" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D89" s="13" t="n">
+        <v>30</v>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>email = min</t>
+          <t>password = max</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
@@ -3800,20 +3775,20 @@
     </row>
     <row r="90">
       <c r="A90" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B90" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C90" s="13" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D90" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>email = min+</t>
+          <t>email = min</t>
         </is>
       </c>
       <c r="F90" s="6" t="inlineStr">
@@ -3834,20 +3809,20 @@
     </row>
     <row r="91">
       <c r="A91" s="4" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B91" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C91" s="13" t="n">
-        <v>149</v>
+        <v>7</v>
       </c>
       <c r="D91" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>email = max-</t>
+          <t>email = min+</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
@@ -3868,20 +3843,20 @@
     </row>
     <row r="92">
       <c r="A92" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B92" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C92" s="13" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D92" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>email = max</t>
+          <t>email = max-</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
@@ -3902,20 +3877,20 @@
     </row>
     <row r="93">
       <c r="A93" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B93" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C93" s="4" t="n">
-        <v>75</v>
+        <v>9</v>
+      </c>
+      <c r="B93" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C93" s="13" t="n">
+        <v>150</v>
       </c>
       <c r="D93" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>fullName = min</t>
+          <t>email = max</t>
         </is>
       </c>
       <c r="F93" s="6" t="inlineStr">
@@ -3936,10 +3911,10 @@
     </row>
     <row r="94">
       <c r="A94" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B94" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C94" s="4" t="n">
         <v>75</v>
@@ -3949,7 +3924,7 @@
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>fullName = min+</t>
+          <t>fullName = min</t>
         </is>
       </c>
       <c r="F94" s="6" t="inlineStr">
@@ -3970,10 +3945,10 @@
     </row>
     <row r="95">
       <c r="A95" s="4" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B95" s="13" t="n">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="C95" s="4" t="n">
         <v>75</v>
@@ -3983,7 +3958,7 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
-          <t>fullName = max-</t>
+          <t>fullName = min+</t>
         </is>
       </c>
       <c r="F95" s="6" t="inlineStr">
@@ -4004,10 +3979,10 @@
     </row>
     <row r="96">
       <c r="A96" s="4" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B96" s="13" t="n">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C96" s="4" t="n">
         <v>75</v>
@@ -4017,118 +3992,119 @@
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
+          <t>fullName = max-</t>
+        </is>
+      </c>
+      <c r="F96" s="6" t="inlineStr">
+        <is>
+          <t>Hợp lệ</t>
+        </is>
+      </c>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H96" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B97" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="C97" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D97" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E97" s="6" t="inlineStr">
+        <is>
           <t>fullName = max</t>
         </is>
       </c>
-      <c r="F96" s="6" t="inlineStr">
+      <c r="F97" s="6" t="inlineStr">
         <is>
           <t>Hợp lệ</t>
         </is>
       </c>
-      <c r="G96" s="6" t="inlineStr">
+      <c r="G97" s="6" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="34" customHeight="1">
-      <c r="A98" s="10" t="inlineStr">
+      <c r="H97" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="34" customHeight="1"/>
+    <row r="99" ht="24" customHeight="1">
+      <c r="A99" s="10" t="inlineStr">
         <is>
           <t>CÁCH ĐỌC: mỗi hàng là MỘT bộ đầy đủ ba biến. Ô tô tím là biến đang được đẩy tới giá trị biên, hai biến còn lại giữ ở nom. Slide 26 nêu nguyên tắc: "tại một thời điểm, BVA chỉ test giá trị biên của 1 biến". Hàng TC3 là bộ tất-cả-nominal, dùng chung cho cả ba biến — đó là lý do công thức là 4n+1 chứ không phải 5n.</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="24" customHeight="1">
-      <c r="A99" s="12" t="inlineStr">
+    <row r="100" ht="30" customHeight="1">
+      <c r="A100" s="12" t="inlineStr">
         <is>
           <t>BẢNG 3 — ROBUSTNESS BVA, phần BỔ SUNG (mẫu slide 24) · 6n + 1 = 19 case</t>
         </is>
       </c>
     </row>
-    <row r="100" ht="30" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B100" s="5" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
+      <c r="C101" s="5" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D100" s="5" t="inlineStr">
+      <c r="D101" s="5" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="E100" s="5" t="inlineStr">
+      <c r="E101" s="5" t="inlineStr">
         <is>
           <t>Biến đang xét</t>
         </is>
       </c>
-      <c r="F100" s="5" t="inlineStr">
+      <c r="F101" s="5" t="inlineStr">
         <is>
           <t>Expected Output</t>
         </is>
       </c>
-      <c r="G100" s="5" t="inlineStr">
+      <c r="G101" s="5" t="inlineStr">
         <is>
           <t>Kết quả thực tế</t>
         </is>
       </c>
-      <c r="H100" s="5" t="inlineStr">
+      <c r="H101" s="5" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B101" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C101" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="D101" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="E101" s="6" t="inlineStr">
-        <is>
-          <t>password = min-</t>
-        </is>
-      </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>KHÔNG hợp lệ</t>
-        </is>
-      </c>
-      <c r="G101" s="6" t="inlineStr">
-        <is>
-          <t>Đúng như mong đợi</t>
-        </is>
-      </c>
-      <c r="H101" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B102" s="4" t="n">
         <v>50</v>
@@ -4137,11 +4113,11 @@
         <v>75</v>
       </c>
       <c r="D102" s="14" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>password = max+</t>
+          <t>password = min-</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
@@ -4162,25 +4138,25 @@
     </row>
     <row r="103">
       <c r="A103" s="4" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B103" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C103" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="D103" s="4" t="n">
-        <v>18</v>
+      <c r="C103" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D103" s="14" t="n">
+        <v>31</v>
       </c>
       <c r="E103" s="6" t="inlineStr">
         <is>
-          <t>email = min-</t>
+          <t>password = max+</t>
         </is>
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>Hợp lệ</t>
+          <t>KHÔNG hợp lệ</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
@@ -4196,25 +4172,25 @@
     </row>
     <row r="104">
       <c r="A104" s="4" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B104" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C104" s="14" t="n">
-        <v>151</v>
+        <v>5</v>
       </c>
       <c r="D104" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
-          <t>email = max+</t>
+          <t>email = min-</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>KHÔNG hợp lệ</t>
+          <t>Hợp lệ</t>
         </is>
       </c>
       <c r="G104" s="6" t="inlineStr">
@@ -4230,20 +4206,20 @@
     </row>
     <row r="105">
       <c r="A105" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B105" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="C105" s="4" t="n">
-        <v>75</v>
+        <v>17</v>
+      </c>
+      <c r="B105" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C105" s="14" t="n">
+        <v>151</v>
       </c>
       <c r="D105" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>fullName = min-</t>
+          <t>email = max+</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
@@ -4264,10 +4240,10 @@
     </row>
     <row r="106">
       <c r="A106" s="4" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B106" s="14" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="C106" s="4" t="n">
         <v>75</v>
@@ -4277,106 +4253,141 @@
       </c>
       <c r="E106" s="6" t="inlineStr">
         <is>
+          <t>fullName = min-</t>
+        </is>
+      </c>
+      <c r="F106" s="6" t="inlineStr">
+        <is>
+          <t>KHÔNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="G106" s="6" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H106" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B107" s="14" t="n">
+        <v>101</v>
+      </c>
+      <c r="C107" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D107" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E107" s="6" t="inlineStr">
+        <is>
           <t>fullName = max+</t>
         </is>
       </c>
-      <c r="F106" s="6" t="inlineStr">
+      <c r="F107" s="6" t="inlineStr">
         <is>
           <t>KHÔNG hợp lệ</t>
         </is>
       </c>
-      <c r="G106" s="6" t="inlineStr">
+      <c r="G107" s="6" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H106" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="34" customHeight="1">
-      <c r="A108" s="10" t="inlineStr">
-        <is>
-          <t>Slide 24: Robustness BVA giữ nguyên phần clean test cases (min, min+, nom, max-, max) và THÊM hai giá trị nằm ngoài miền hợp lệ là min- và max+. Mười ba case ở bảng 2 cộng sáu case ở đây là 19 = 6n + 1.</t>
-        </is>
-      </c>
-    </row>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="34" customHeight="1"/>
     <row r="109" ht="34" customHeight="1">
       <c r="A109" s="10" t="inlineStr">
         <is>
+          <t>Slide 24: Robustness BVA giữ nguyên phần clean test cases (min, min+, nom, max-, max) và THÊM hai giá trị nằm ngoài miền hợp lệ là min- và max+. Mười ba case ở bảng 2 cộng sáu case ở đây là 19 = 6n + 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="10" t="inlineStr">
+        <is>
           <t>PHÁT HIỆN Ở TC16: theo thiết kế, email 5 ký tự (min-) phải bị từ chối. Thực tế được CHẤP NHẬN, vì @Size của email chỉ khai max=150, không khai min. Đã kiểm chứng thêm: "a@b" (3 ký tự) cũng hợp lệ. Đây là chênh lệch giữa biên giả định và ràng buộc thực tế trong mã nguồn, không phải lỗi của test.</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="24" customHeight="1">
-      <c r="A110" s="12" t="inlineStr">
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="12" t="inlineStr">
         <is>
           <t>BẢNG 4 — PHÂN HOẠCH LỚP TƯƠNG ĐƯƠNG (mẫu slide 32)</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="30" customHeight="1">
-      <c r="A111" s="5" t="inlineStr">
+    <row r="112" ht="62" customHeight="1">
+      <c r="A112" s="5" t="inlineStr">
         <is>
           <t>Conditions</t>
         </is>
       </c>
-      <c r="B111" s="5" t="inlineStr">
+      <c r="B112" s="5" t="inlineStr">
         <is>
           <t>Valid Partitions</t>
         </is>
       </c>
-      <c r="C111" s="5" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="D111" s="5" t="inlineStr">
+      <c r="D112" s="5" t="inlineStr">
         <is>
           <t>Invalid Partitions</t>
         </is>
       </c>
-      <c r="E111" s="5" t="inlineStr">
+      <c r="E112" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="F111" s="5" t="inlineStr">
+      <c r="F112" s="5" t="inlineStr">
         <is>
           <t>Valid Boundaries</t>
         </is>
       </c>
-      <c r="G111" s="5" t="inlineStr">
+      <c r="G112" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="H111" s="5" t="inlineStr">
+      <c r="H112" s="5" t="inlineStr">
         <is>
           <t>Robustness</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="62" customHeight="1">
-      <c r="A112" s="6" t="inlineStr">
+    <row r="113" ht="62" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B112" s="6" t="inlineStr">
+      <c r="B113" s="6" t="inlineStr">
         <is>
           <t>6–30 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C112" s="6" t="inlineStr">
+      <c r="C113" s="6" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
+      <c r="D113" s="6" t="inlineStr">
         <is>
           <t>&lt; 6 ký tự
 &gt; 30 ký tự
@@ -4384,7 +4395,7 @@
 null</t>
         </is>
       </c>
-      <c r="E112" s="6" t="inlineStr">
+      <c r="E113" s="6" t="inlineStr">
         <is>
           <t>X1
 X2
@@ -4392,223 +4403,225 @@
 X4</t>
         </is>
       </c>
-      <c r="F112" s="6" t="inlineStr">
+      <c r="F113" s="6" t="inlineStr">
         <is>
           <t>6, 7, 18, 29, 30</t>
         </is>
       </c>
-      <c r="G112" s="6" t="inlineStr">
+      <c r="G113" s="6" t="inlineStr">
         <is>
           <t>B1–B5</t>
         </is>
       </c>
-      <c r="H112" s="6" t="inlineStr">
+      <c r="H113" s="6" t="inlineStr">
         <is>
           <t>5 và 31 (B6, B7)</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="62" customHeight="1">
-      <c r="A113" s="6" t="inlineStr">
+    <row r="114" ht="62" customHeight="1">
+      <c r="A114" s="6" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="B113" s="6" t="inlineStr">
+      <c r="B114" s="6" t="inlineStr">
         <is>
           <t>1–100 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C113" s="6" t="inlineStr">
+      <c r="C114" s="6" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="D113" s="6" t="inlineStr">
+      <c r="D114" s="6" t="inlineStr">
         <is>
           <t>&gt; 100 ký tự
 toàn khoảng trắng
 null</t>
         </is>
       </c>
-      <c r="E113" s="6" t="inlineStr">
+      <c r="E114" s="6" t="inlineStr">
         <is>
           <t>X5
 X6
 X7</t>
         </is>
       </c>
-      <c r="F113" s="6" t="inlineStr">
+      <c r="F114" s="6" t="inlineStr">
         <is>
           <t>1, 2, 50, 99, 100</t>
         </is>
       </c>
-      <c r="G113" s="6" t="inlineStr">
+      <c r="G114" s="6" t="inlineStr">
         <is>
           <t>B8–B12</t>
         </is>
       </c>
-      <c r="H113" s="6" t="inlineStr">
+      <c r="H114" s="6" t="inlineStr">
         <is>
           <t>rỗng (= min−1) và 101
 (B13, B14)</t>
         </is>
       </c>
     </row>
-    <row r="114" ht="62" customHeight="1">
-      <c r="A114" s="6" t="inlineStr">
+    <row r="115" ht="62" customHeight="1">
+      <c r="A115" s="6" t="inlineStr">
         <is>
           <t>email — điều kiện ĐỘ DÀI</t>
         </is>
       </c>
-      <c r="B114" s="6" t="inlineStr">
+      <c r="B115" s="6" t="inlineStr">
         <is>
           <t>≤ 150 ký tự</t>
         </is>
       </c>
-      <c r="C114" s="6" t="inlineStr">
+      <c r="C115" s="6" t="inlineStr">
         <is>
           <t>V3</t>
         </is>
       </c>
-      <c r="D114" s="6" t="inlineStr">
+      <c r="D115" s="6" t="inlineStr">
         <is>
           <t>&gt; 150 ký tự</t>
         </is>
       </c>
-      <c r="E114" s="6" t="inlineStr">
+      <c r="E115" s="6" t="inlineStr">
         <is>
           <t>X9</t>
         </is>
       </c>
-      <c r="F114" s="6" t="inlineStr">
+      <c r="F115" s="6" t="inlineStr">
         <is>
           <t>75, 149, 150
 (KHÔNG có biên dưới)</t>
         </is>
       </c>
-      <c r="G114" s="6" t="inlineStr">
+      <c r="G115" s="6" t="inlineStr">
         <is>
           <t>B15–B17</t>
         </is>
       </c>
-      <c r="H114" s="6" t="inlineStr">
+      <c r="H115" s="6" t="inlineStr">
         <is>
           <t>151 (B18, chỉ có max+)</t>
         </is>
       </c>
     </row>
-    <row r="115" ht="62" customHeight="1">
-      <c r="A115" s="6" t="inlineStr">
+    <row r="116" ht="62" customHeight="1">
+      <c r="A116" s="6" t="inlineStr">
         <is>
           <t>email — điều kiện ĐỊNH DẠNG</t>
         </is>
       </c>
-      <c r="B115" s="6" t="inlineStr">
+      <c r="B116" s="6" t="inlineStr">
         <is>
           <t>đúng định dạng email</t>
         </is>
       </c>
-      <c r="C115" s="6" t="inlineStr">
+      <c r="C116" s="6" t="inlineStr">
         <is>
           <t>V4</t>
         </is>
       </c>
-      <c r="D115" s="6" t="inlineStr">
+      <c r="D116" s="6" t="inlineStr">
         <is>
           <t>sai định dạng
 null / rỗng</t>
         </is>
       </c>
-      <c r="E115" s="6" t="inlineStr">
+      <c r="E116" s="6" t="inlineStr">
         <is>
           <t>X8
 X10</t>
         </is>
       </c>
-      <c r="F115" s="6" t="inlineStr">
+      <c r="F116" s="6" t="inlineStr">
         <is>
           <t>(không áp dụng —
 miền rời rạc)</t>
         </is>
       </c>
-      <c r="G115" s="6" t="inlineStr">
+      <c r="G116" s="6" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H115" s="6" t="inlineStr">
+      <c r="H116" s="6" t="inlineStr">
         <is>
           <t>(không áp dụng)</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="62" customHeight="1">
-      <c r="A116" s="6" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="6" t="inlineStr">
         <is>
           <t>Tệp bảng điểm — DUNG LƯỢNG</t>
         </is>
       </c>
-      <c r="B116" s="6" t="inlineStr">
+      <c r="B117" s="6" t="inlineStr">
         <is>
           <t>0 đến 10 MB</t>
         </is>
       </c>
-      <c r="C116" s="6" t="inlineStr">
+      <c r="C117" s="6" t="inlineStr">
         <is>
           <t>V5</t>
         </is>
       </c>
-      <c r="D116" s="6" t="inlineStr">
+      <c r="D117" s="6" t="inlineStr">
         <is>
           <t>&gt; 10 MB</t>
         </is>
       </c>
-      <c r="E116" s="6" t="inlineStr">
+      <c r="E117" s="6" t="inlineStr">
         <is>
           <t>X11</t>
         </is>
       </c>
-      <c r="F116" s="6" t="inlineStr">
+      <c r="F117" s="6" t="inlineStr">
         <is>
           <t>0, 1 byte, 5 MB,
 10MB−1, 10 MB</t>
         </is>
       </c>
-      <c r="G116" s="6" t="inlineStr">
+      <c r="G117" s="6" t="inlineStr">
         <is>
           <t>B19–B23</t>
         </is>
       </c>
-      <c r="H116" s="6" t="inlineStr">
+      <c r="H117" s="6" t="inlineStr">
         <is>
           <t>10MB + 1 byte (B24)</t>
         </is>
       </c>
     </row>
-    <row r="118" ht="34" customHeight="1">
-      <c r="A118" s="10" t="inlineStr">
-        <is>
-          <t>Slide 32 gộp phân lớp tương đương và giá trị biên vào MỘT bảng. Một trường có thể mang nhiều dòng điều kiện độc lập — trường Customer name ở slide 29 được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email ở đây cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên, còn điều kiện ĐỊNH DẠNG là miền rời rạc nên chỉ phân lớp được.</t>
-        </is>
-      </c>
-    </row>
+    <row r="118" ht="34" customHeight="1"/>
     <row r="119" ht="34" customHeight="1">
       <c r="A119" s="10" t="inlineStr">
         <is>
+          <t>Slide 32 gộp phân lớp tương đương và giá trị biên vào MỘT bảng. Một trường có thể mang nhiều dòng điều kiện độc lập — trường Customer name ở slide 29 được tách thành 'độ dài 2–64' và 'ký tự hợp lệ'. Email ở đây cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên, còn điều kiện ĐỊNH DẠNG là miền rời rạc nên chỉ phân lớp được.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="10" t="inlineStr">
+        <is>
           <t>PHÁT HIỆN — lớp X3: mật khẩu 8 dấu cách có độ dài 8, THOẢ MÃN @Size(min=6, max=30) nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện được.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A109:H109"/>
     <mergeCell ref="A5:H5"/>
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A73:H73"/>
+    <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A82:H82"/>
     <mergeCell ref="A99:H99"/>
-    <mergeCell ref="A82:H82"/>
     <mergeCell ref="A98:H98"/>
     <mergeCell ref="A108:H108"/>
     <mergeCell ref="A118:H118"/>

</xml_diff>

<commit_message>
docs(report): thêm Bảng 5 - thiết kế test case gộp tag theo mẫu slide 33
Báo cáo trước đây dừng ở slide 32 (bảng phân lớp + biên có gắn tag V/X/B) mà
thiếu bước cuối của ví dụ Loan application: gộp các tag đó thành test case.

Bảng 5 dựng 22 case phủ trọn 40 tag (V1-V5, X1-X11, B1-B24), cột New Tags
Covered ghi tag phủ lần đầu như slide 33:
  TC1-TC5    case hợp lệ, mỗi case gộp nhiều tag vì không trường nào che trường nào
  TC6-TC16   case không hợp lệ, mỗi case đúng MỘT vi phạm để tránh che lỗi
  TC17-TC22  tệp bảng điểm, tách riêng vì không thuộc form đăng ký

Vài case không hợp lệ phủ hai tag do giá trị biên nằm trong lớp không hợp lệ,
ví dụ TC6 password = 5 ký tự phủ cả X1 (< 6) lẫn B6 (min-1).
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -62,7 +62,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +104,11 @@
         <fgColor rgb="00FBE4E4"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -131,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,6 +176,18 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -537,7 +554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H120"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4613,10 +4630,726 @@
         </is>
       </c>
     </row>
+    <row r="122" ht="24" customHeight="1">
+      <c r="A122" s="15" t="inlineStr">
+        <is>
+          <t>BẢNG 5 — THIẾT KẾ TEST CASE, GỘP TAG (mẫu slide 33) · 22 case phủ trọn 40 tag</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="5" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Input</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>Expected Outcome</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
+        <is>
+          <t>New Tags Covered</t>
+        </is>
+      </c>
+      <c r="E123" s="5" t="inlineStr"/>
+      <c r="F123" s="5" t="inlineStr"/>
+      <c r="G123" s="5" t="inlineStr"/>
+      <c r="H123" s="5" t="inlineStr">
+        <is>
+          <t>Test đã thi hành</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="46" customHeight="1">
+      <c r="A124" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 1 ký tự
+email = 75 ký tự
+password = 6 ký tự</t>
+        </is>
+      </c>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công</t>
+        </is>
+      </c>
+      <c r="D124" s="17" t="inlineStr">
+        <is>
+          <t>V1, V2, V3, V4,
+B1, B8, B15</t>
+        </is>
+      </c>
+      <c r="E124" s="6" t="inlineStr"/>
+      <c r="F124" s="6" t="inlineStr"/>
+      <c r="G124" s="6" t="inlineStr"/>
+      <c r="H124" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="46" customHeight="1">
+      <c r="A125" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 2 ký tự
+email = 149 ký tự
+password = 7 ký tự</t>
+        </is>
+      </c>
+      <c r="C125" s="6" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công</t>
+        </is>
+      </c>
+      <c r="D125" s="17" t="inlineStr">
+        <is>
+          <t>B2, B9, B16</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="inlineStr"/>
+      <c r="F125" s="6" t="inlineStr"/>
+      <c r="G125" s="6" t="inlineStr"/>
+      <c r="H125" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="46" customHeight="1">
+      <c r="A126" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 50 ký tự
+email = 150 ký tự
+password = 18 ký tự</t>
+        </is>
+      </c>
+      <c r="C126" s="6" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công</t>
+        </is>
+      </c>
+      <c r="D126" s="17" t="inlineStr">
+        <is>
+          <t>B3, B10, B17</t>
+        </is>
+      </c>
+      <c r="E126" s="6" t="inlineStr"/>
+      <c r="F126" s="6" t="inlineStr"/>
+      <c r="G126" s="6" t="inlineStr"/>
+      <c r="H126" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="46" customHeight="1">
+      <c r="A127" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="B127" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 99 ký tự
+email = 75 ký tự
+password = 29 ký tự</t>
+        </is>
+      </c>
+      <c r="C127" s="6" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công</t>
+        </is>
+      </c>
+      <c r="D127" s="17" t="inlineStr">
+        <is>
+          <t>B4, B11</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="inlineStr"/>
+      <c r="F127" s="6" t="inlineStr"/>
+      <c r="G127" s="6" t="inlineStr"/>
+      <c r="H127" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="46" customHeight="1">
+      <c r="A128" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B128" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 100 ký tự
+email = 75 ký tự
+password = 30 ký tự</t>
+        </is>
+      </c>
+      <c r="C128" s="6" t="inlineStr">
+        <is>
+          <t>Đăng ký thành công</t>
+        </is>
+      </c>
+      <c r="D128" s="17" t="inlineStr">
+        <is>
+          <t>B5, B12</t>
+        </is>
+      </c>
+      <c r="E128" s="6" t="inlineStr"/>
+      <c r="F128" s="6" t="inlineStr"/>
+      <c r="G128" s="6" t="inlineStr"/>
+      <c r="H128" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="46" customHeight="1">
+      <c r="A129" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>password = 5 ký tự
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C129" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — password phải ≥ 6 ký tự</t>
+        </is>
+      </c>
+      <c r="D129" s="19" t="inlineStr">
+        <is>
+          <t>X1, B6</t>
+        </is>
+      </c>
+      <c r="E129" s="6" t="inlineStr"/>
+      <c r="F129" s="6" t="inlineStr"/>
+      <c r="G129" s="6" t="inlineStr"/>
+      <c r="H129" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="46" customHeight="1">
+      <c r="A130" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>password = 31 ký tự
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C130" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — password phải ≤ 30 ký tự</t>
+        </is>
+      </c>
+      <c r="D130" s="19" t="inlineStr">
+        <is>
+          <t>X2, B7</t>
+        </is>
+      </c>
+      <c r="E130" s="6" t="inlineStr"/>
+      <c r="F130" s="6" t="inlineStr"/>
+      <c r="G130" s="6" t="inlineStr"/>
+      <c r="H130" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="46" customHeight="1">
+      <c r="A131" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>password = 8 dấu cách
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C131" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — password không được để trống</t>
+        </is>
+      </c>
+      <c r="D131" s="19" t="inlineStr">
+        <is>
+          <t>X3</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="inlineStr"/>
+      <c r="F131" s="6" t="inlineStr"/>
+      <c r="G131" s="6" t="inlineStr"/>
+      <c r="H131" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="46" customHeight="1">
+      <c r="A132" s="18" t="n">
+        <v>9</v>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>password = null
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C132" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — password bắt buộc</t>
+        </is>
+      </c>
+      <c r="D132" s="19" t="inlineStr">
+        <is>
+          <t>X4</t>
+        </is>
+      </c>
+      <c r="E132" s="6" t="inlineStr"/>
+      <c r="F132" s="6" t="inlineStr"/>
+      <c r="G132" s="6" t="inlineStr"/>
+      <c r="H132" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="46" customHeight="1">
+      <c r="A133" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 101 ký tự
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C133" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — họ tên phải ≤ 100 ký tự</t>
+        </is>
+      </c>
+      <c r="D133" s="19" t="inlineStr">
+        <is>
+          <t>X5, B14</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="inlineStr"/>
+      <c r="F133" s="6" t="inlineStr"/>
+      <c r="G133" s="6" t="inlineStr"/>
+      <c r="H133" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="46" customHeight="1">
+      <c r="A134" s="18" t="n">
+        <v>11</v>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>fullName = 5 dấu cách
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C134" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — họ tên không được để trống</t>
+        </is>
+      </c>
+      <c r="D134" s="19" t="inlineStr">
+        <is>
+          <t>X6</t>
+        </is>
+      </c>
+      <c r="E134" s="6" t="inlineStr"/>
+      <c r="F134" s="6" t="inlineStr"/>
+      <c r="G134" s="6" t="inlineStr"/>
+      <c r="H134" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="46" customHeight="1">
+      <c r="A135" s="18" t="n">
+        <v>12</v>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>fullName = null
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C135" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — họ tên bắt buộc</t>
+        </is>
+      </c>
+      <c r="D135" s="19" t="inlineStr">
+        <is>
+          <t>X7</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="inlineStr"/>
+      <c r="F135" s="6" t="inlineStr"/>
+      <c r="G135" s="6" t="inlineStr"/>
+      <c r="H135" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="46" customHeight="1">
+      <c r="A136" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>fullName = chuỗi rỗng
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C136" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — họ tên không được để trống</t>
+        </is>
+      </c>
+      <c r="D136" s="19" t="inlineStr">
+        <is>
+          <t>B13</t>
+        </is>
+      </c>
+      <c r="E136" s="6" t="inlineStr"/>
+      <c r="F136" s="6" t="inlineStr"/>
+      <c r="G136" s="6" t="inlineStr"/>
+      <c r="H136" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="46" customHeight="1">
+      <c r="A137" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>email = "khong-phai-email"
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C137" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — email sai định dạng</t>
+        </is>
+      </c>
+      <c r="D137" s="19" t="inlineStr">
+        <is>
+          <t>X8</t>
+        </is>
+      </c>
+      <c r="E137" s="6" t="inlineStr"/>
+      <c r="F137" s="6" t="inlineStr"/>
+      <c r="G137" s="6" t="inlineStr"/>
+      <c r="H137" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="46" customHeight="1">
+      <c r="A138" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B138" s="6" t="inlineStr">
+        <is>
+          <t>email = 151 ký tự
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C138" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — email phải ≤ 150 ký tự</t>
+        </is>
+      </c>
+      <c r="D138" s="19" t="inlineStr">
+        <is>
+          <t>X9, B18</t>
+        </is>
+      </c>
+      <c r="E138" s="6" t="inlineStr"/>
+      <c r="F138" s="6" t="inlineStr"/>
+      <c r="G138" s="6" t="inlineStr"/>
+      <c r="H138" s="6" t="inlineStr">
+        <is>
+          <t>RegisterFormDTOBvaTest
+RegisterStandardBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="46" customHeight="1">
+      <c r="A139" s="18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B139" s="6" t="inlineStr">
+        <is>
+          <t>email = null
+(hai trường kia hợp lệ)</t>
+        </is>
+      </c>
+      <c r="C139" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — email bắt buộc</t>
+        </is>
+      </c>
+      <c r="D139" s="19" t="inlineStr">
+        <is>
+          <t>X10</t>
+        </is>
+      </c>
+      <c r="E139" s="6" t="inlineStr"/>
+      <c r="F139" s="6" t="inlineStr"/>
+      <c r="G139" s="6" t="inlineStr"/>
+      <c r="H139" s="6" t="inlineStr">
+        <is>
+          <t>RegisterEquivalencePartitionTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="46" customHeight="1">
+      <c r="A140" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B140" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 0 byte</t>
+        </is>
+      </c>
+      <c r="C140" s="6" t="inlineStr">
+        <is>
+          <t>Tải lên thành công</t>
+        </is>
+      </c>
+      <c r="D140" s="17" t="inlineStr">
+        <is>
+          <t>V5, B19</t>
+        </is>
+      </c>
+      <c r="E140" s="6" t="inlineStr"/>
+      <c r="F140" s="6" t="inlineStr"/>
+      <c r="G140" s="6" t="inlineStr"/>
+      <c r="H140" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="46" customHeight="1">
+      <c r="A141" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B141" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 1 byte</t>
+        </is>
+      </c>
+      <c r="C141" s="6" t="inlineStr">
+        <is>
+          <t>Tải lên thành công</t>
+        </is>
+      </c>
+      <c r="D141" s="17" t="inlineStr">
+        <is>
+          <t>B20</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="inlineStr"/>
+      <c r="F141" s="6" t="inlineStr"/>
+      <c r="G141" s="6" t="inlineStr"/>
+      <c r="H141" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="46" customHeight="1">
+      <c r="A142" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 5 MB</t>
+        </is>
+      </c>
+      <c r="C142" s="6" t="inlineStr">
+        <is>
+          <t>Tải lên thành công</t>
+        </is>
+      </c>
+      <c r="D142" s="17" t="inlineStr">
+        <is>
+          <t>B21</t>
+        </is>
+      </c>
+      <c r="E142" s="6" t="inlineStr"/>
+      <c r="F142" s="6" t="inlineStr"/>
+      <c r="G142" s="6" t="inlineStr"/>
+      <c r="H142" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="46" customHeight="1">
+      <c r="A143" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 10 MB − 1 byte</t>
+        </is>
+      </c>
+      <c r="C143" s="6" t="inlineStr">
+        <is>
+          <t>Tải lên thành công</t>
+        </is>
+      </c>
+      <c r="D143" s="17" t="inlineStr">
+        <is>
+          <t>B22</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="inlineStr"/>
+      <c r="F143" s="6" t="inlineStr"/>
+      <c r="G143" s="6" t="inlineStr"/>
+      <c r="H143" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="46" customHeight="1">
+      <c r="A144" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 10 MB</t>
+        </is>
+      </c>
+      <c r="C144" s="6" t="inlineStr">
+        <is>
+          <t>Tải lên thành công</t>
+        </is>
+      </c>
+      <c r="D144" s="17" t="inlineStr">
+        <is>
+          <t>B23</t>
+        </is>
+      </c>
+      <c r="E144" s="6" t="inlineStr"/>
+      <c r="F144" s="6" t="inlineStr"/>
+      <c r="G144" s="6" t="inlineStr"/>
+      <c r="H144" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="46" customHeight="1">
+      <c r="A145" s="18" t="n">
+        <v>22</v>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>Tệp bảng điểm = 10 MB + 1 byte</t>
+        </is>
+      </c>
+      <c r="C145" s="6" t="inlineStr">
+        <is>
+          <t>Từ chối — tệp vượt quá 10 MB</t>
+        </is>
+      </c>
+      <c r="D145" s="19" t="inlineStr">
+        <is>
+          <t>X11, B24</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="inlineStr"/>
+      <c r="F145" s="6" t="inlineStr"/>
+      <c r="G145" s="6" t="inlineStr"/>
+      <c r="H145" s="6" t="inlineStr">
+        <is>
+          <t>OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="40" customHeight="1">
+      <c r="A147" s="10" t="inlineStr">
+        <is>
+          <t>CÁCH ĐỌC: mỗi hàng là MỘT lần điền form đầy đủ rồi bấm gửi, giống bảng "Thiết kế test cases" ở slide 33. Cột New Tags Covered ghi những tag mà case đó phủ LẦN ĐẦU — tag đã phủ ở case trước thì không ghi lại. Nền xanh = case hợp lệ, nền hồng = case bị từ chối.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="40" customHeight="1">
+      <c r="A148" s="10" t="inlineStr">
+        <is>
+          <t>VÌ SAO CHỈ CẦN 22 CASE CHO 40 TAG: case HỢP LỆ được phép gộp nhiều tag cùng lúc — TC1 vừa phủ V1 V2 V3 V4 vừa phủ ba giá trị biên B1 B8 B15, vì cả ba trường đều hợp lệ nên không trường nào che kết quả của trường nào. Ngược lại case KHÔNG hợp lệ chỉ được đặt MỘT vi phạm mỗi lần: nếu vừa để password quá ngắn vừa để email sai định dạng thì form vẫn báo lỗi, nhưng không biết nó bắt được vi phạm nào — hiện tượng che lỗi (masking). Vì vậy 11 tag X phải trải ra 11 case riêng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="40" customHeight="1">
+      <c r="A149" s="10" t="inlineStr">
+        <is>
+          <t>GỘP THÊM ĐỂ TỐI THIỂU HOÁ: vài case không hợp lệ phủ được hai tag cùng lúc vì giá trị biên nằm ngay trong lớp không hợp lệ. TC6 đặt password = 5 ký tự nên vừa phủ lớp X1 (&lt; 6 ký tự) vừa phủ giá trị biên B6 (min−1). TC7, TC10, TC15, TC22 cũng theo cách này.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="40" customHeight="1">
+      <c r="A150" s="10" t="inlineStr">
+        <is>
+          <t>TC17–TC22 tách riêng vì tệp bảng điểm KHÔNG thuộc form đăng ký — nó là chức năng tải bảng điểm ở bước onboarding. Slide 33 gộp tag trong phạm vi MỘT màn hình nhập liệu, hai chức năng khác nhau thì không gộp chung một lần submit được.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="17">
+    <mergeCell ref="A122:H122"/>
     <mergeCell ref="A109:H109"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A147:H147"/>
+    <mergeCell ref="A148:H148"/>
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A73:H73"/>
     <mergeCell ref="A72:H72"/>
@@ -4625,8 +5358,10 @@
     <mergeCell ref="A98:H98"/>
     <mergeCell ref="A108:H108"/>
     <mergeCell ref="A118:H118"/>
+    <mergeCell ref="A150:H150"/>
     <mergeCell ref="A110:H110"/>
     <mergeCell ref="A119:H119"/>
+    <mergeCell ref="A149:H149"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs(report): bảng tổng kết sheet 01 chỉ giữ lớp test bám mẫu slide
Bỏ RegisterFormDTOBvaTest khỏi bảng tổng kết, còn 4 dòng / 54 test. File vẫn nằm
trong source, chỉ không xuất hiện trong báo cáo.

Lý do: nó chia mỗi trường thành một test case riêng, mà slide chưa bao giờ trình
bày test case ở dạng đó. Slide 29-31 chỉ là bước PHÂN TÍCH biên theo từng trường,
rồi gom vào bảng tag slide 32; mọi TEST CASE trong slide - cả 23 lẫn 33 - đều là
một bộ đầu vào đầy đủ. Giữ nó trong báo cáo thì phải giải thích một dạng bảng
không có trong bài giảng.

Không mất độ phủ: B1-B18 đã được RegisterStandardBvaTest kiểm qua Bảng 2, 3 và
RegisterTagCoverageTest kiểm qua Bảng 5. Ghi rõ ánh xạ này ở ghi chú dưới Bảng 4.
</commit_message>
<xml_diff>
--- a/BaoCao-PhanA-HopDen.xlsx
+++ b/BaoCao-PhanA-HopDen.xlsx
@@ -596,7 +596,7 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>TỔNG KẾT THI HÀNH — 81 test đã chạy, 81 PASS, 0 fail. Mỗi dòng là một lớp test trong source, cột cuối chỉ ra nó thi hành bảng nào.</t>
+          <t>TỔNG KẾT THI HÀNH — 54 test đã chạy, 54 PASS, 0 fail. Mỗi dòng là một lớp test trong source, cột cuối chỉ ra nó thi hành bảng nào.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,8 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Bảng 2, Bảng 3</t>
+          <t>Bảng 2, Bảng 3
+Bảng 4 · B1–B18</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr"/>
@@ -689,20 +690,20 @@
     <row r="8" ht="32" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>RegisterFormDTOBvaTest</t>
+          <t>RegisterEquivalencePartitionTest</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>BVA theo từng trường</t>
+          <t>Phân hoạch lớp tương đương</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Bảng 4 · B1–B18</t>
+          <t>Bảng 4 · V1–V4, X1–X10</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
@@ -717,20 +718,21 @@
     <row r="9" ht="32" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>RegisterEquivalencePartitionTest</t>
+          <t>OnboardingFileSizeBvaTest</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Phân hoạch lớp tương đương</t>
+          <t>BVA dung lượng tệp</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Bảng 4 · V1–V4, X1–X10</t>
+          <t>Bảng 4 · V5, B19–B24
+Bảng 5 · TC17–TC22</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr"/>
@@ -742,278 +744,283 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>OnboardingFileSizeBvaTest</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>TỔNG</t>
+        </is>
+      </c>
+      <c r="B10" s="22" t="n">
+        <v>54</v>
+      </c>
+      <c r="C10" s="21" t="inlineStr"/>
+      <c r="D10" s="21" t="inlineStr"/>
+      <c r="E10" s="21" t="inlineStr"/>
+      <c r="F10" s="21" t="inlineStr"/>
+      <c r="G10" s="21" t="inlineStr"/>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Số ở cột "Số test" được đối chiếu tự động với target/surefire-reports khi sinh lại sheet này bằng tools/gen_sheet01.py — nếu source chạy ra số khác thì script dừng và báo lỗi, nên báo cáo không thể lệch với code. Chạy lại để kiểm chứng: mvnw test -Dtest=RegisterStandardBvaTest,RegisterTagCoverageTest,RegisterEquivalencePartitionTest,OnboardingFileSizeBvaTest</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>BẢNG 1 — ĐỊNH NGHĨA GIÁ TRỊ BIÊN CỦA TỪNG BIẾN (phần ghi chú bên trái slide 23)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Giá trị</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>fullName (số ký tự)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>email (số ký tự)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>password (số ký tự)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>min</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>BVA dung lượng tệp</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Bảng 4 · V5, B19–B24
-Bảng 5 · TC17–TC22</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="6" t="inlineStr"/>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>TỔNG</t>
-        </is>
-      </c>
-      <c r="B11" s="22" t="n">
-        <v>81</v>
-      </c>
-      <c r="C11" s="21" t="inlineStr"/>
-      <c r="D11" s="21" t="inlineStr"/>
-      <c r="E11" s="21" t="inlineStr"/>
-      <c r="F11" s="21" t="inlineStr"/>
-      <c r="G11" s="21" t="inlineStr"/>
-      <c r="H11" s="23" t="inlineStr">
-        <is>
-          <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Số ở cột "Số test" được đối chiếu tự động với target/surefire-reports khi sinh lại sheet này bằng tools/gen_sheet01.py — nếu source chạy ra số khác thì script dừng và báo lỗi, nên báo cáo không thể lệch với code. Chạy lại để kiểm chứng: mvnw test -Dtest=RegisterStandardBvaTest,RegisterTagCoverageTest,RegisterFormDTOBvaTest,RegisterEquivalencePartitionTest,OnboardingFileSizeBvaTest</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>BẢNG 1 — ĐỊNH NGHĨA GIÁ TRỊ BIÊN CỦA TỪNG BIẾN (phần ghi chú bên trái slide 23)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Giá trị</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>fullName (số ký tự)</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>email (số ký tự)</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>password (số ký tự)</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
+      <c r="D15" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>giá trị nhỏ nhất hợp lệ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>min</t>
+          <t>min+</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E16" s="6" t="inlineStr"/>
       <c r="F16" s="6" t="inlineStr"/>
       <c r="G16" s="6" t="inlineStr"/>
       <c r="H16" s="6" t="inlineStr">
         <is>
-          <t>giá trị nhỏ nhất hợp lệ</t>
+          <t>ngay trên min</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>min+</t>
+          <t>nom</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="6" t="inlineStr"/>
       <c r="G17" s="6" t="inlineStr"/>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>ngay trên min</t>
+          <t>giá trị điển hình, giữa miền</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>nom</t>
+          <t>max-</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>75</v>
+        <v>149</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="E18" s="6" t="inlineStr"/>
       <c r="F18" s="6" t="inlineStr"/>
       <c r="G18" s="6" t="inlineStr"/>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>giá trị điển hình, giữa miền</t>
+          <t>ngay dưới max</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>max-</t>
+          <t>max</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="6" t="inlineStr"/>
       <c r="G19" s="6" t="inlineStr"/>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>ngay dưới max</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>150</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="E20" s="6" t="inlineStr"/>
-      <c r="F20" s="6" t="inlineStr"/>
-      <c r="G20" s="6" t="inlineStr"/>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
           <t>giá trị lớn nhất hợp lệ</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Ràng buộc gốc: fullName @NotBlank @Size(max=100) · email @NotBlank @Email @Size(max=150) · password @NotBlank @Size(min=6, max=30). Biên dưới của fullName do @NotBlank sinh ra (chuỗi rỗng bị chặn nên min = 1). Biên dưới của email là BIÊN VẬN HÀNH — độ dài email quy ước ngắn nhất a@b.co — vì @Size không khai min.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="15" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>BẢNG 2 — STANDARD BVA TEST CASES (mẫu slide 23) · số case = 4n + 1 = 4×3 + 1 = 13</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Case</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="E24" s="5" t="inlineStr">
+      <c r="E23" s="5" t="inlineStr">
         <is>
           <t>Biến đang xét</t>
         </is>
       </c>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="F23" s="5" t="inlineStr">
         <is>
           <t>Expected Output</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>Kết quả thực tế</t>
         </is>
       </c>
-      <c r="H24" s="5" t="inlineStr">
+      <c r="H23" s="5" t="inlineStr">
         <is>
           <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="D24" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>password = min</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Hợp lệ</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>Đúng như mong đợi</t>
+        </is>
+      </c>
+      <c r="H24" s="7" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B25" s="4" t="n">
         <v>50</v>
@@ -1022,11 +1029,11 @@
         <v>75</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>password = min</t>
+          <t>password = min+</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
@@ -1047,7 +1054,7 @@
     </row>
     <row r="26">
       <c r="A26" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B26" s="4" t="n">
         <v>50</v>
@@ -1055,12 +1062,12 @@
       <c r="C26" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D26" s="13" t="n">
-        <v>7</v>
+      <c r="D26" s="4" t="n">
+        <v>18</v>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>password = min+</t>
+          <t>TẤT CẢ nominal</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
@@ -1081,7 +1088,7 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B27" s="4" t="n">
         <v>50</v>
@@ -1089,12 +1096,12 @@
       <c r="C27" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D27" s="4" t="n">
-        <v>18</v>
+      <c r="D27" s="13" t="n">
+        <v>29</v>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>TẤT CẢ nominal</t>
+          <t>password = max-</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
@@ -1115,7 +1122,7 @@
     </row>
     <row r="28">
       <c r="A28" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B28" s="4" t="n">
         <v>50</v>
@@ -1124,11 +1131,11 @@
         <v>75</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>password = max-</t>
+          <t>password = max</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
@@ -1149,20 +1156,20 @@
     </row>
     <row r="29">
       <c r="A29" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B29" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C29" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="D29" s="13" t="n">
-        <v>30</v>
+      <c r="C29" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="D29" s="4" t="n">
+        <v>18</v>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>password = max</t>
+          <t>email = min</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -1183,20 +1190,20 @@
     </row>
     <row r="30">
       <c r="A30" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B30" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C30" s="13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>email = min</t>
+          <t>email = min+</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr">
@@ -1217,20 +1224,20 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B31" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C31" s="13" t="n">
-        <v>7</v>
+        <v>149</v>
       </c>
       <c r="D31" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>email = min+</t>
+          <t>email = max-</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -1251,20 +1258,20 @@
     </row>
     <row r="32">
       <c r="A32" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B32" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C32" s="13" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>email = max-</t>
+          <t>email = max</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -1285,20 +1292,20 @@
     </row>
     <row r="33">
       <c r="A33" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>150</v>
+        <v>10</v>
+      </c>
+      <c r="B33" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>75</v>
       </c>
       <c r="D33" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>email = max</t>
+          <t>fullName = min</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -1319,10 +1326,10 @@
     </row>
     <row r="34">
       <c r="A34" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>75</v>
@@ -1332,7 +1339,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>fullName = min</t>
+          <t>fullName = min+</t>
         </is>
       </c>
       <c r="F34" s="6" t="inlineStr">
@@ -1353,10 +1360,10 @@
     </row>
     <row r="35">
       <c r="A35" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B35" s="13" t="n">
-        <v>2</v>
+        <v>99</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>75</v>
@@ -1366,7 +1373,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>fullName = min+</t>
+          <t>fullName = max-</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -1387,10 +1394,10 @@
     </row>
     <row r="36">
       <c r="A36" s="4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B36" s="13" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C36" s="4" t="n">
         <v>75</v>
@@ -1400,7 +1407,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>fullName = max-</t>
+          <t>fullName = max</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -1419,99 +1426,99 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B37" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="C37" s="4" t="n">
+    <row r="37" ht="40" customHeight="1">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>CÁCH ĐỌC: mỗi hàng là MỘT bộ đầy đủ ba biến. Ô tô tím là biến đang được đẩy tới giá trị biên, hai biến còn lại giữ ở nom. Slide 26 nêu nguyên tắc: tại một thời điểm, BVA chỉ test giá trị biên của 1 biến. Hàng TC3 là bộ tất-cả-nominal, dùng chung cho cả ba biến — đó là lý do công thức là 4n+1 chứ không phải 5n. Code: RegisterStandardBvaTest · standardBva_moiBoDeuHopLe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="24" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>BẢNG 3 — ROBUSTNESS BVA, phần BỔ SUNG (mẫu slide 24) · 6n + 1 = 19 case</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Case</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>fullName</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>password</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Biến đang xét</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Expected Output</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>Kết quả thực tế</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C41" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="D37" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E37" s="6" t="inlineStr">
-        <is>
-          <t>fullName = max</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
-        <is>
-          <t>Hợp lệ</t>
-        </is>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="D41" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="E41" s="6" t="inlineStr">
+        <is>
+          <t>password = min-</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>KHÔNG hợp lệ</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>Đúng như mong đợi</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>PASS</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="40" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>CÁCH ĐỌC: mỗi hàng là MỘT bộ đầy đủ ba biến. Ô tô tím là biến đang được đẩy tới giá trị biên, hai biến còn lại giữ ở nom. Slide 26 nêu nguyên tắc: tại một thời điểm, BVA chỉ test giá trị biên của 1 biến. Hàng TC3 là bộ tất-cả-nominal, dùng chung cho cả ba biến — đó là lý do công thức là 4n+1 chứ không phải 5n. Code: RegisterStandardBvaTest · standardBva_moiBoDeuHopLe.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
-        <is>
-          <t>BẢNG 3 — ROBUSTNESS BVA, phần BỔ SUNG (mẫu slide 24) · 6n + 1 = 19 case</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="30" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>Case</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>fullName</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>password</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Biến đang xét</t>
-        </is>
-      </c>
-      <c r="F41" s="5" t="inlineStr">
-        <is>
-          <t>Expected Output</t>
-        </is>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>Kết quả thực tế</t>
-        </is>
-      </c>
-      <c r="H41" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B42" s="4" t="n">
         <v>50</v>
@@ -1520,11 +1527,11 @@
         <v>75</v>
       </c>
       <c r="D42" s="14" t="n">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>password = min-</t>
+          <t>password = max+</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
@@ -1545,25 +1552,25 @@
     </row>
     <row r="43">
       <c r="A43" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B43" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="C43" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="D43" s="14" t="n">
-        <v>31</v>
+      <c r="C43" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" s="4" t="n">
+        <v>18</v>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>password = max+</t>
+          <t>email = min-</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>KHÔNG hợp lệ</t>
+          <t>Hợp lệ</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -1579,25 +1586,25 @@
     </row>
     <row r="44">
       <c r="A44" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B44" s="4" t="n">
         <v>50</v>
       </c>
       <c r="C44" s="14" t="n">
-        <v>5</v>
+        <v>151</v>
       </c>
       <c r="D44" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>email = min-</t>
+          <t>email = max+</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>Hợp lệ</t>
+          <t>KHÔNG hợp lệ</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -1613,20 +1620,20 @@
     </row>
     <row r="45">
       <c r="A45" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B45" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="C45" s="14" t="n">
-        <v>151</v>
+        <v>18</v>
+      </c>
+      <c r="B45" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="4" t="n">
+        <v>75</v>
       </c>
       <c r="D45" s="4" t="n">
         <v>18</v>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>email = max+</t>
+          <t>fullName = min-</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -1647,10 +1654,10 @@
     </row>
     <row r="46">
       <c r="A46" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B46" s="14" t="n">
-        <v>0</v>
+        <v>101</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>75</v>
@@ -1660,7 +1667,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>fullName = min-</t>
+          <t>fullName = max+</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -1679,121 +1686,87 @@
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B47" s="14" t="n">
-        <v>101</v>
-      </c>
-      <c r="C47" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="D47" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="E47" s="6" t="inlineStr">
-        <is>
-          <t>fullName = max+</t>
-        </is>
-      </c>
-      <c r="F47" s="6" t="inlineStr">
-        <is>
-          <t>KHÔNG hợp lệ</t>
-        </is>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>Đúng như mong đợi</t>
-        </is>
-      </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>PASS</t>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>Slide 24: Robustness BVA giữ nguyên phần clean test cases (min, min+, nom, max-, max) và THÊM hai giá trị nằm ngoài miền hợp lệ là min- và max+. Mười ba case ở Bảng 2 cộng sáu case ở đây là 19 = 6n + 1. Code: RegisterStandardBvaTest · robustnessBva_giaTriNgoaiBien.</t>
         </is>
       </c>
     </row>
     <row r="48" ht="40" customHeight="1">
       <c r="A48" s="10" t="inlineStr">
         <is>
-          <t>Slide 24: Robustness BVA giữ nguyên phần clean test cases (min, min+, nom, max-, max) và THÊM hai giá trị nằm ngoài miền hợp lệ là min- và max+. Mười ba case ở Bảng 2 cộng sáu case ở đây là 19 = 6n + 1. Code: RegisterStandardBvaTest · robustnessBva_giaTriNgoaiBien.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="40" customHeight="1">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
           <t>PHÁT HIỆN Ở TC16: theo thiết kế, email 5 ký tự (min-) phải bị từ chối. Thực tế được CHẤP NHẬN, vì @Size của email chỉ khai max=150, không khai min. Đã kiểm chứng thêm: a@b (3 ký tự) cũng hợp lệ. Đây là chênh lệch giữa biên giả định và ràng buộc thực tế trong mã nguồn, không phải lỗi của test.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="24" customHeight="1">
-      <c r="A51" s="15" t="inlineStr">
+    <row r="50" ht="24" customHeight="1">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>BẢNG 4 — PHÂN HOẠCH LỚP TƯƠNG ĐƯƠNG (mẫu slide 32)</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="30" customHeight="1">
-      <c r="A52" s="5" t="inlineStr">
+    <row r="51" ht="30" customHeight="1">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Conditions</t>
         </is>
       </c>
-      <c r="B52" s="5" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>Valid Partitions</t>
         </is>
       </c>
-      <c r="C52" s="5" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Invalid Partitions</t>
         </is>
       </c>
-      <c r="E52" s="5" t="inlineStr">
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="F52" s="5" t="inlineStr">
+      <c r="F51" s="5" t="inlineStr">
         <is>
           <t>Valid Boundaries</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>Tag</t>
         </is>
       </c>
-      <c r="H52" s="5" t="inlineStr">
+      <c r="H51" s="5" t="inlineStr">
         <is>
           <t>Robustness</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="62" customHeight="1">
-      <c r="A53" s="6" t="inlineStr">
+    <row r="52" ht="62" customHeight="1">
+      <c r="A52" s="6" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="B53" s="6" t="inlineStr">
+      <c r="B52" s="6" t="inlineStr">
         <is>
           <t>6–30 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C53" s="6" t="inlineStr">
+      <c r="C52" s="6" t="inlineStr">
         <is>
           <t>V1</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>&lt; 6 ký tự
 &gt; 30 ký tự
@@ -1801,7 +1774,7 @@
 null</t>
         </is>
       </c>
-      <c r="E53" s="6" t="inlineStr">
+      <c r="E52" s="6" t="inlineStr">
         <is>
           <t>X1
 X2
@@ -1809,212 +1782,219 @@
 X4</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="F52" s="6" t="inlineStr">
         <is>
           <t>6, 7, 18, 29, 30</t>
         </is>
       </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>B1–B5</t>
         </is>
       </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>5 và 31 (B6, B7)</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="62" customHeight="1">
-      <c r="A54" s="6" t="inlineStr">
+    <row r="53" ht="62" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
         <is>
           <t>fullName</t>
         </is>
       </c>
-      <c r="B54" s="6" t="inlineStr">
+      <c r="B53" s="6" t="inlineStr">
         <is>
           <t>1–100 ký tự,
 có ít nhất 1 ký tự không trắng</t>
         </is>
       </c>
-      <c r="C54" s="6" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>V2</t>
         </is>
       </c>
-      <c r="D54" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>&gt; 100 ký tự
 toàn khoảng trắng
 null</t>
         </is>
       </c>
-      <c r="E54" s="6" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>X5
 X6
 X7</t>
         </is>
       </c>
-      <c r="F54" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
         <is>
           <t>1, 2, 50, 99, 100</t>
         </is>
       </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="G53" s="6" t="inlineStr">
         <is>
           <t>B8–B12</t>
         </is>
       </c>
-      <c r="H54" s="6" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>rỗng (= min−1) và 101
 (B13, B14)</t>
         </is>
       </c>
     </row>
+    <row r="54" ht="62" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>email — điều kiện ĐỘ DÀI</t>
+        </is>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>≤ 150 ký tự</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>V3</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr">
+        <is>
+          <t>&gt; 150 ký tự</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>X9</t>
+        </is>
+      </c>
+      <c r="F54" s="6" t="inlineStr">
+        <is>
+          <t>75, 149, 150
+(KHÔNG có biên dưới)</t>
+        </is>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>B15–B17</t>
+        </is>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
+        <is>
+          <t>151 (B18, chỉ có max+)</t>
+        </is>
+      </c>
+    </row>
     <row r="55" ht="62" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>email — điều kiện ĐỘ DÀI</t>
+          <t>email — điều kiện ĐỊNH DẠNG</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>≤ 150 ký tự</t>
+          <t>đúng định dạng email</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>V3</t>
+          <t>V4</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>&gt; 150 ký tự</t>
+          <t>sai định dạng
+null / rỗng</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>X9</t>
+          <t>X8
+X10</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>75, 149, 150
-(KHÔNG có biên dưới)</t>
+          <t>(không áp dụng —
+miền rời rạc)</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>B15–B17</t>
+          <t>–</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>151 (B18, chỉ có max+)</t>
+          <t>(không áp dụng)</t>
         </is>
       </c>
     </row>
     <row r="56" ht="62" customHeight="1">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>email — điều kiện ĐỊNH DẠNG</t>
+          <t>Tệp bảng điểm — DUNG LƯỢNG</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>đúng định dạng email</t>
+          <t>0 đến 10 MB</t>
         </is>
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>V4</t>
+          <t>V5</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>sai định dạng
-null / rỗng</t>
+          <t>&gt; 10 MB</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>X8
-X10</t>
+          <t>X11</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
-        <is>
-          <t>(không áp dụng —
-miền rời rạc)</t>
-        </is>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="H56" s="6" t="inlineStr">
-        <is>
-          <t>(không áp dụng)</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="62" customHeight="1">
-      <c r="A57" s="6" t="inlineStr">
-        <is>
-          <t>Tệp bảng điểm — DUNG LƯỢNG</t>
-        </is>
-      </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>0 đến 10 MB</t>
-        </is>
-      </c>
-      <c r="C57" s="6" t="inlineStr">
-        <is>
-          <t>V5</t>
-        </is>
-      </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>&gt; 10 MB</t>
-        </is>
-      </c>
-      <c r="E57" s="6" t="inlineStr">
-        <is>
-          <t>X11</t>
-        </is>
-      </c>
-      <c r="F57" s="6" t="inlineStr">
         <is>
           <t>0, 1 byte, 5 MB,
 10MB−1, 10 MB</t>
         </is>
       </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="G56" s="6" t="inlineStr">
         <is>
           <t>B19–B23</t>
         </is>
       </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>10MB + 1 byte (B24)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="40" customHeight="1">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>Slide 32 gộp phân lớp tương đương và giá trị biên vào MỘT bảng. Một trường có thể mang nhiều dòng điều kiện độc lập — trường Customer name ở slide 29 được tách thành độ dài 2-64 và ký tự hợp lệ. Email ở đây cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên, còn điều kiện ĐỊNH DẠNG là miền rời rạc nên chỉ phân lớp được — đó là ý nghĩa của dấu "-" ở cột Tag dòng thứ tư.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="40" customHeight="1">
       <c r="A58" s="10" t="inlineStr">
         <is>
-          <t>Slide 32 gộp phân lớp tương đương và giá trị biên vào MỘT bảng. Một trường có thể mang nhiều dòng điều kiện độc lập — trường Customer name ở slide 29 được tách thành độ dài 2-64 và ký tự hợp lệ. Email ở đây cũng vậy: điều kiện ĐỘ DÀI có thứ tự nên áp được giá trị biên, còn điều kiện ĐỊNH DẠNG là miền rời rạc nên chỉ phân lớp được — đó là ý nghĩa của dấu "-" ở cột Tag dòng thứ tư.</t>
+          <t>CODE KIỂM CHỨNG BẢNG NÀY: cột Valid/Invalid Partitions do RegisterEquivalencePartitionTest kiểm; cột Valid Boundaries B1–B18 do RegisterStandardBvaTest kiểm (xem Bảng 2, Bảng 3); B19–B24 của tệp bảng điểm do OnboardingFileSizeBvaTest kiểm.</t>
         </is>
       </c>
     </row>
     <row r="59" ht="40" customHeight="1">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>PHÁT HIỆN — lớp X3: mật khẩu 8 dấu cách có độ dài 8, THOẢ MÃN @Size(min=6, max=30) nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện được. Code: RegisterEquivalencePartitionTest.</t>
+          <t>PHÁT HIỆN — lớp X3: mật khẩu 8 dấu cách có độ dài 8, THOẢ MÃN @Size(min=6, max=30) nhưng vẫn bị @NotBlank từ chối. Lớp này không nằm ở ranh giới độ dài nào nên giá trị biên không chạm tới — chỉ phân hoạch lớp tương đương mới phát hiện được. Code: RegisterEquivalencePartitionTest · x3_toanKhoangTrang_biTuChoi.</t>
         </is>
       </c>
     </row>
@@ -2751,25 +2731,26 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="A12:H12"/>
+  <mergeCells count="19">
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A39:H39"/>
+    <mergeCell ref="A59:H59"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A88:H88"/>
+    <mergeCell ref="A87:H87"/>
+    <mergeCell ref="A37:H37"/>
+    <mergeCell ref="A89:H89"/>
+    <mergeCell ref="A50:H50"/>
+    <mergeCell ref="A86:H86"/>
+    <mergeCell ref="A57:H57"/>
+    <mergeCell ref="A85:H85"/>
+    <mergeCell ref="A47:H47"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A86:H86"/>
-    <mergeCell ref="A87:H87"/>
-    <mergeCell ref="A59:H59"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A51:H51"/>
-    <mergeCell ref="A85:H85"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A89:H89"/>
-    <mergeCell ref="A61:H61"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A58:H58"/>
-    <mergeCell ref="A88:H88"/>
-    <mergeCell ref="A40:H40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>